<commit_message>
Updates based on crosschecks
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-BCS.xlsx
+++ b/baseline/data_processing_elements-BCS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\OneDrive\Bureau\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480A0186-A116-4638-B809-5EDADB665E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EA421D2-20A5-4FB3-BFFD-D1609871F519}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="1001">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="1005">
   <si>
     <t>index</t>
   </si>
@@ -2315,75 +2315,6 @@
 Hours spent reading-weekend.  Self-reported questionnaire "How many hours do you spend reading books (including in electronic format, e.g. Kindle) at home? b) On a typical day at the weekend". Options were: None,  Less than an hour a day, 1 to 2 hours a day, 2 to 3 hours a day, 3 to 4 hours a day,  More than 4 hours a day</t>
   </si>
   <si>
-    <t xml:space="preserve">case_when(
-(rowSums(mutate(.,
-temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
-B10Q15A == 2 ~ 0.5*5;
-B10Q15A == 3 ~ 1.5*5;
-B10Q15A == 4 ~ 2.5*5;
-B10Q15A == 5 ~ 3.5*5;
-B10Q15A == 6 ~ 4*5;
-ELSE ~ NA_real_),
-temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
-B10Q15B == 2 ~ 0.5*2;
-B10Q15B == 3 ~ 1.5*2;
-B10Q15B == 4 ~ 2.5*2;
-B10Q15B == 5 ~ 3.5*2;
-B10Q15B == 6 ~ 4*2;
-ELSE ~ NA_real_)) %&gt;%
-select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt; 1 ~ 1L;
-(rowSums(mutate(.,
-temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
-B10Q15A == 2 ~ 0.5*5;
-B10Q15A == 3 ~ 1.5*5;
-B10Q15A == 4 ~ 2.5*5;
-B10Q15A == 5 ~ 3.5*5;
-B10Q15A == 6 ~ 4*5;
-ELSE ~ NA_real_),
-temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
-B10Q15B == 2 ~ 0.5*2;
-B10Q15B == 3 ~ 1.5*2;
-B10Q15B == 4 ~ 2.5*2;
-B10Q15B == 5 ~ 3.5*2;
-B10Q15B == 6 ~ 4*2;
-ELSE ~ NA_real_)) %&gt;%
-select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt;= 1 &amp;
-(rowSums(mutate(.,
-temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
-B10Q15A == 2 ~ 0.5*5;
-B10Q15A == 3 ~ 1.5*5;
-B10Q15A == 4 ~ 2.5*5;
-B10Q15A == 5 ~ 3.5*5;
-B10Q15A == 6 ~ 4*5;
-ELSE ~ NA_real_),
-temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
-B10Q15B == 2 ~ 0.5*2;
-B10Q15B == 3 ~ 1.5*2;
-B10Q15B == 4 ~ 2.5*2;
-B10Q15B == 5 ~ 3.5*2;
-B10Q15B == 6 ~ 4*2;
-ELSE ~ NA_real_)) %&gt;%
-select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt;= 3 ~ 2L;
-(rowSums(mutate(.,
-temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
-B10Q15A == 2 ~ 0.5*5;
-B10Q15A == 3 ~ 1.5*5;
-B10Q15A == 4 ~ 2.5*5;
-B10Q15A == 5 ~ 3.5*5;
-B10Q15A == 6 ~ 4*5;
-ELSE ~ NA_real_),
-temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
-B10Q15B == 2 ~ 0.5*2;
-B10Q15B == 3 ~ 1.5*2;
-B10Q15B == 4 ~ 2.5*2;
-B10Q15B == 5 ~ 3.5*2;
-B10Q15B == 6 ~ 4*2;
-ELSE ~ NA_real_)) %&gt;%
-select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt; 3 ~ 3L; 
-ELSE ~ NA_integer_)
-</t>
-  </si>
-  <si>
     <t>lsb_sed_beh_total_sitting</t>
   </si>
   <si>
@@ -3996,21 +3927,6 @@
   </si>
   <si>
     <t>There is an option for None of the above. Coded Presumed no based on this.</t>
-  </si>
-  <si>
-    <t>case_when(
-  B10KHPB10 == 1 |
-    rowSums(across(matches("B10LNGDRC4_|BDRC4_"), ~ .x == 205)) &gt; 0 ~ 1L;
-  B10KHPB10 == 0 &amp;
-    rowSums(across(matches("B10LNGDRC4_|BDRC4_"), ~ .x %in% c(-9, -8, -1, 205))) == 0 ~ 0L;
-  B10KHPB10 == 0 &amp;
-    rowSums(across(matches("B10LNGDRC4_|BDRC4_"), ~ .x %in% c(-9, -8, -1, 205))) &gt; 0 ~ 2L;
-  B10KHPB10 %in% c(-9, -8, -1) &amp;
-    rowSums(across(matches("B10LNGDRC4_|B10DRC4_"), ~ .x %in% c(-9, -8, -1, 205))) == 0 ~ 2L;
-  ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
-    <t>Change starts_with to matches (cannot use | with starts_with).</t>
   </si>
   <si>
     <t>Unclear what -1 Not applicable is, but doesn't affect many participants.</t>
@@ -4436,19 +4352,6 @@
 BNF code subchapter</t>
   </si>
   <si>
-    <t>All study-specific medication values matching drugs under BNF section 2.12 (lipid-regulating drugs) were coded as lipid-lowering. 
-Any reported medication with relevant drug code was coded as 1=Yes (question wording implied current medications) regardless of whether it was taken in the last period.
-Study-specific medication datast was converted from long to wide in pre-processing.</t>
-  </si>
-  <si>
-    <t>Rewrote algorithm with if_any for simplicity/readability.
-Code no based on responses to B10MEDCN: whether taking any medicines and B10MEDLN: any long-acting medication, otherwise NA. 
-Removed condition that long-acting medication used in last period (this ranges from one week to 5 years) and add harmo comment. The question wording implies current medication. 
-Changed coding of NA to use drug code variables instead of taken in last period, to include non long-acting meds, and only use Refused, Not known (not Not applicable).
-Added comment about coding of lipid-regulating drugs. 
-Medication variables converted from long to wide in pre-processing.</t>
-  </si>
-  <si>
     <t>case_when(
 B10MEDCN == 2 &amp; B10MEDLN == 2 ~ 0L ; 
 if_any(c(B10LNGDRC4_1, B10LNGDRC4_2, B10LNGDRC4_3, B10LNGDRC4_4, B10LNGDRC4_5, B10LNGDRC4_6, B10LNGDRC4_7, B10LNGDRC4_8, B10LNGDRC4_9, B10LNGDRC4_10, B10DRC4_1, B10DRC4_2, B10DRC4_3, B10DRC4_4, B10DRC4_5, B10DRC4_6, B10DRC4_7, B10DRC4_8, B10DRC4_9, B10DRC4_10), ~ .x == 212) ~ 1L;
@@ -4502,15 +4405,7 @@
     <t xml:space="preserve">(Derived) SF-36 Physical functioning score  </t>
   </si>
   <si>
-    <t>There is a derived study variable available.</t>
-  </si>
-  <si>
     <t xml:space="preserve">(-8) Not enough information    </t>
-  </si>
-  <si>
-    <t>case_when(
-BD10PHHE &gt;= 0 ~ as.numeric(BD10PHHE);
-ELSE ~ NA_real_)</t>
   </si>
   <si>
     <t>Type of heart prob since last int/4 yrs: Coronary heart disease ; 
@@ -4761,6 +4656,152 @@
   </si>
   <si>
     <t>Updated to presume no for anyone that didn't select high blood pressure, heart problems, or stroke. Previous rule was much more conservative.</t>
+  </si>
+  <si>
+    <t>All study-specific medication values matching drugs under BNF section 205.0 (Hypertension and Heart Failure) were coded as medication use. 
+Any reported medication with relevant drug code was coded as 1=Yes (question wording implied current medications) regardless of whether it was taken in the last period.
+Study-specific medication datast was converted from long to wide in pre-processing.</t>
+  </si>
+  <si>
+    <t>All study-specific medication values matching drugs under BNF section 2.12 (lipid-regulating drugs) were coded as medication use. 
+Any reported medication with relevant drug code was coded as 1=Yes (question wording implied current medications) regardless of whether it was taken in the last period.
+Study-specific medication datast was converted from long to wide in pre-processing.</t>
+  </si>
+  <si>
+    <t>All study-specific medication values matching drugs under BNF section 601.0 (Drugs Used In Diabetes) were coded as medication use. 
+Any reported medication with relevant drug code was coded as 1=Yes (question wording implied current medications) regardless of whether it was taken in the last period.
+Study-specific medication datast was converted from long to wide in pre-processing.</t>
+  </si>
+  <si>
+    <t>Rewrote algorithm with if_any for simplicity/readability.
+Code no based on responses to B10MEDCN: whether taking any medicines and B10MEDLN: any long-acting medication, otherwise NA. 
+Removed condition that long-acting medication used in last period (this ranges from one week to 5 years) and add harmo comment. The question wording implies current medication. 
+Changed coding of NA to use drug code variables instead of taken in last period, to include non long-acting meds, and only use Refused, Not known (not Not applicable).
+Added comment about coding of medication use. 
+Medication variables converted from long to wide in pre-processing.</t>
+  </si>
+  <si>
+    <t>Rewrote algorithm with if_any for simplicity/readability.
+Code now based on responses to B10MEDCN: whether taking any medicines and B10MEDLN: any long-acting medication, otherwise NA. 
+Removed condition that long-acting medication used in last period (this ranges from one week to 5 years) and add harmo comment. The question wording implies current medication. 
+Changed coding of NA to use drug code variables instead of taken in last period, to include non long-acting meds, and only use Refused, Not known (not Not applicable).
+Added comment about coding of medication use. 
+Medication variables converted from long to wide in pre-processing.
+Additional update: Fixed harmo comment referring to lipid-lowering drugs.</t>
+  </si>
+  <si>
+    <t>Rewrote algorithm with if_any for simplicity/readability.
+Code no based on responses to B10MEDCN: whether taking any medicines and B10MEDLN: any long-acting medication, otherwise NA. 
+Removed condition that long-acting medication used in last period (this ranges from one week to 5 years) and add harmo comment. The question wording implies current medication. 
+Changed coding of NA to use drug code variables instead of taken in last period, to include non long-acting meds, and only use Refused, Not known (not Not applicable).
+Added comment about coding of medication use. 
+Medication variables converted from long to wide in pre-processing.
+Additional update: Fixed harmo comment referring to lipid-lowering drugs.</t>
+  </si>
+  <si>
+    <t>case_when(
+  B10KHPB10 == 1 ~ 1L ; 
+  if_any(c(B10LNGDRC4_1, B10LNGDRC4_2, B10LNGDRC4_3, B10LNGDRC4_4, B10LNGDRC4_5, B10LNGDRC4_6, B10LNGDRC4_7, B10LNGDRC4_8, B10LNGDRC4_9, B10LNGDRC4_10, B10DRC4_1, B10DRC4_2, B10DRC4_3, B10DRC4_4, B10DRC4_5, B10DRC4_6, B10DRC4_7, B10DRC4_8, B10DRC4_9, B10DRC4_10), ~ .x == 205) ~ 1L ;
+  B10KHPB10 == 0 &amp; B10MEDCN == 2 &amp; B10MEDLN == 2 ~ 0L ; 
+  B10KHPB10 == 0 ~ 2L ; 
+  if_all(c(B10LNGDRC4_1, B10LNGDRC4_2, B10LNGDRC4_3, B10LNGDRC4_4, B10LNGDRC4_5, B10LNGDRC4_6, B10LNGDRC4_7, B10LNGDRC4_8, B10LNGDRC4_9, B10LNGDRC4_10, B10DRC4_1, B10DRC4_2, B10DRC4_3, B10DRC4_4, B10DRC4_5, B10DRC4_6, B10DRC4_7, B10DRC4_8, B10DRC4_9, B10DRC4_10), ~ !.x  %in% c(-9, -8) &amp; !is.na(.x)) ~ 2L ; 
+  ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>Change starts_with to matches (cannot use | with starts_with).
+Additional updates based on cross-checks for consistency with medication use.</t>
+  </si>
+  <si>
+    <t>There is a derived study variable available.
+Additional updates based on crosschecks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">case_when(
+(rowSums(mutate(.,
+temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
+B10Q15A == 2 ~ 0.5*5;
+B10Q15A == 3 ~ 1.5*5;
+B10Q15A == 4 ~ 2.5*5;
+B10Q15A == 5 ~ 3.5*5;
+B10Q15A == 6 ~ 4*5;
+ELSE ~ NA_real_),
+temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
+B10Q15B == 2 ~ 0.5*2;
+B10Q15B == 3 ~ 1.5*2;
+B10Q15B == 4 ~ 2.5*2;
+B10Q15B == 5 ~ 3.5*2;
+B10Q15B == 6 ~ 4*2;
+ELSE ~ NA_real_)) %&gt;%
+select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt; 1 ~ 1L;
+(rowSums(mutate(.,
+temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
+B10Q15A == 2 ~ 0.5*5;
+B10Q15A == 3 ~ 1.5*5;
+B10Q15A == 4 ~ 2.5*5;
+B10Q15A == 5 ~ 3.5*5;
+B10Q15A == 6 ~ 4*5;
+ELSE ~ NA_real_),
+temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
+B10Q15B == 2 ~ 0.5*2;
+B10Q15B == 3 ~ 1.5*2;
+B10Q15B == 4 ~ 2.5*2;
+B10Q15B == 5 ~ 3.5*2;
+B10Q15B == 6 ~ 4*2;
+ELSE ~ NA_real_)) %&gt;%
+select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt;= 1 &amp;
+(rowSums(mutate(.,
+temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
+B10Q15A == 2 ~ 0.5*5;
+B10Q15A == 3 ~ 1.5*5;
+B10Q15A == 4 ~ 2.5*5;
+B10Q15A == 5 ~ 3.5*5;
+B10Q15A == 6 ~ 4*5;
+ELSE ~ NA_real_),
+temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
+B10Q15B == 2 ~ 0.5*2;
+B10Q15B == 3 ~ 1.5*2;
+B10Q15B == 4 ~ 2.5*2;
+B10Q15B == 5 ~ 3.5*2;
+B10Q15B == 6 ~ 4*2;
+ELSE ~ NA_real_)) %&gt;%
+select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt;= 3 ~ 2L;
+(rowSums(mutate(.,
+temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;
+B10Q15A == 2 ~ 0.5*5;
+B10Q15A == 3 ~ 1.5*5;
+B10Q15A == 4 ~ 2.5*5;
+B10Q15A == 5 ~ 3.5*5;
+B10Q15A == 6 ~ 4*5;
+ELSE ~ NA_real_),
+temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;
+B10Q15B == 2 ~ 0.5*2;
+B10Q15B == 3 ~ 1.5*2;
+B10Q15B == 4 ~ 2.5*2;
+B10Q15B == 5 ~ 3.5*2;
+B10Q15B == 6 ~ 4*2;
+ELSE ~ NA_real_)) %&gt;%
+select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt; 3 ~ 3L; 
+ELSE ~ NA_integer_)
+</t>
+  </si>
+  <si>
+    <t>case_when(
+rowSums(mutate(.,
+temp_B10Q2A = if_else(!B10Q2A %in% c(1, 2, 3), NA, 1), 
+temp_B10Q2B = if_else(!B10Q2B %in% c(1, 2, 3), NA, 1),
+temp_B10Q2C = if_else(!B10Q2C %in% c(1, 2, 3), NA, 1),
+temp_B10Q2D = if_else(!B10Q2D %in% c(1, 2, 3), NA, 1),
+temp_B10Q2E = if_else(!B10Q2E %in% c(1, 2, 3), NA, 1),
+temp_B10Q2F = if_else(!B10Q2F %in% c(1, 2, 3), NA, 1),
+temp_B10Q2G = if_else(!B10Q2G %in% c(1, 2, 3), NA, 1),
+temp_B10Q2H = if_else(!B10Q2H %in% c(1, 2, 3), NA, 1),
+temp_B10Q2I = if_else(!B10Q2I %in% c(1, 2, 3), NA, 1),
+temp_B10Q2J = if_else(!B10Q2J %in% c(1, 2, 3), NA, 1)) %&gt;%
+select(temp_B10Q2A, temp_B10Q2B, temp_B10Q2C, temp_B10Q2D, temp_B10Q2E,
+temp_B10Q2F, temp_B10Q2G, temp_B10Q2H, temp_B10Q2I, temp_B10Q2J), 
+na.rm = TRUE) &lt; 5 ~ NA_real_ ; 
+BD10PHHE &gt;= 0 ~ as.numeric(BD10PHHE);
+ELSE ~ NA_real_)</t>
   </si>
 </sst>
 </file>
@@ -5319,6 +5360,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AG122"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5452,7 +5494,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17">
         <v>1</v>
       </c>
@@ -5505,7 +5547,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17">
         <v>2</v>
       </c>
@@ -5546,7 +5588,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17">
         <v>3</v>
       </c>
@@ -5587,10 +5629,10 @@
         <v>59</v>
       </c>
       <c r="AC4" s="22" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17">
         <v>4</v>
       </c>
@@ -5628,7 +5670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:33" ht="210" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17">
         <v>5</v>
       </c>
@@ -5681,7 +5723,7 @@
         <v>78</v>
       </c>
       <c r="V6" s="22" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>44</v>
@@ -5699,7 +5741,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="17">
         <v>6</v>
       </c>
@@ -5752,7 +5794,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:33" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -5805,16 +5847,16 @@
         <v>45</v>
       </c>
       <c r="Y8" s="24" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="Z8" s="24" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="AC8" s="18" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
     </row>
-    <row r="9" spans="1:33" ht="180" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17">
         <v>8</v>
       </c>
@@ -5864,7 +5906,7 @@
         <v>116</v>
       </c>
       <c r="V9" s="22" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>44</v>
@@ -5876,22 +5918,22 @@
         <v>92</v>
       </c>
       <c r="Z9" s="14" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>117</v>
       </c>
       <c r="AB9" s="23" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="AC9" s="22" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="AD9" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
-    <row r="10" spans="1:33" ht="165" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="17">
         <v>9</v>
       </c>
@@ -5953,16 +5995,16 @@
         <v>122</v>
       </c>
       <c r="AB10" s="23" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="AC10" s="22" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="AD10" s="23" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
-    <row r="11" spans="1:33" ht="285" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="17">
         <v>10</v>
       </c>
@@ -6015,7 +6057,7 @@
         <v>134</v>
       </c>
       <c r="V11" s="22" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>44</v>
@@ -6030,7 +6072,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:33" ht="285" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="17">
         <v>11</v>
       </c>
@@ -6083,7 +6125,7 @@
         <v>134</v>
       </c>
       <c r="V12" s="22" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>44</v>
@@ -6098,7 +6140,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:33" ht="255" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="17">
         <v>12</v>
       </c>
@@ -6151,7 +6193,7 @@
         <v>134</v>
       </c>
       <c r="V13" s="22" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>147</v>
@@ -6166,7 +6208,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="14" spans="1:33" ht="285" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="17">
         <v>13</v>
       </c>
@@ -6219,7 +6261,7 @@
         <v>134</v>
       </c>
       <c r="V14" s="22" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>44</v>
@@ -6237,10 +6279,10 @@
         <v>155</v>
       </c>
       <c r="AC14" s="18" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
-    <row r="15" spans="1:33" ht="285" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="17">
         <v>14</v>
       </c>
@@ -6293,7 +6335,7 @@
         <v>134</v>
       </c>
       <c r="V15" s="22" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>44</v>
@@ -6305,13 +6347,13 @@
         <v>92</v>
       </c>
       <c r="Z15" s="14" t="s">
+        <v>834</v>
+      </c>
+      <c r="AC15" s="22" t="s">
         <v>835</v>
       </c>
-      <c r="AC15" s="22" t="s">
-        <v>836</v>
-      </c>
     </row>
-    <row r="16" spans="1:33" ht="285" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17">
         <v>15</v>
       </c>
@@ -6364,7 +6406,7 @@
         <v>134</v>
       </c>
       <c r="V16" s="22" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>44</v>
@@ -6376,13 +6418,13 @@
         <v>92</v>
       </c>
       <c r="Z16" s="14" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="AC16" s="22" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
     </row>
-    <row r="17" spans="1:30" ht="255" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="17">
         <v>16</v>
       </c>
@@ -6435,7 +6477,7 @@
         <v>134</v>
       </c>
       <c r="V17" s="22" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="W17" s="16" t="s">
         <v>147</v>
@@ -6450,7 +6492,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="18" spans="1:30" ht="255" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="17">
         <v>17</v>
       </c>
@@ -6503,7 +6545,7 @@
         <v>134</v>
       </c>
       <c r="V18" s="22" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="W18" s="16" t="s">
         <v>147</v>
@@ -6518,7 +6560,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="19" spans="1:30" ht="285" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" ht="285" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="17">
         <v>18</v>
       </c>
@@ -6571,7 +6613,7 @@
         <v>134</v>
       </c>
       <c r="V19" s="22" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="W19" s="16" t="s">
         <v>44</v>
@@ -6586,7 +6628,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="20" spans="1:30" ht="195" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="17">
         <v>19</v>
       </c>
@@ -6636,7 +6678,7 @@
         <v>194</v>
       </c>
       <c r="V20" s="22" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="W20" s="25" t="s">
         <v>44</v>
@@ -6653,10 +6695,10 @@
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
       <c r="AC20" s="22" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
     </row>
-    <row r="21" spans="1:30" ht="195" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17">
         <v>20</v>
       </c>
@@ -6706,7 +6748,7 @@
         <v>194</v>
       </c>
       <c r="V21" s="22" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="W21" s="16" t="s">
         <v>44</v>
@@ -6721,7 +6763,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="22" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="17">
         <v>21</v>
       </c>
@@ -6744,13 +6786,13 @@
         <v>206</v>
       </c>
       <c r="M22" s="18" t="s">
+        <v>846</v>
+      </c>
+      <c r="N22" s="18" t="s">
         <v>847</v>
       </c>
-      <c r="N22" s="18" t="s">
+      <c r="T22" s="22" t="s">
         <v>848</v>
-      </c>
-      <c r="T22" s="22" t="s">
-        <v>849</v>
       </c>
       <c r="W22" s="24" t="s">
         <v>44</v>
@@ -6762,16 +6804,16 @@
         <v>81</v>
       </c>
       <c r="Z22" s="22" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AB22" s="22" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="AD22" s="22" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
     </row>
-    <row r="23" spans="1:30" ht="255" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" ht="255" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="17">
         <v>22</v>
       </c>
@@ -6827,7 +6869,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="24" spans="1:30" ht="195" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="17">
         <v>23</v>
       </c>
@@ -6886,7 +6928,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="25" spans="1:30" ht="150" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="17">
         <v>24</v>
       </c>
@@ -6927,7 +6969,7 @@
         <v>232</v>
       </c>
       <c r="V25" s="22" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="W25" s="16" t="s">
         <v>44</v>
@@ -6942,13 +6984,13 @@
         <v>233</v>
       </c>
       <c r="AA25" s="18" t="s">
+        <v>850</v>
+      </c>
+      <c r="AC25" s="22" t="s">
         <v>851</v>
       </c>
-      <c r="AC25" s="22" t="s">
-        <v>852</v>
-      </c>
     </row>
-    <row r="26" spans="1:30" ht="180" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17">
         <v>25</v>
       </c>
@@ -7001,7 +7043,7 @@
         <v>246</v>
       </c>
       <c r="V26" s="22" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="W26" s="16" t="s">
         <v>44</v>
@@ -7016,10 +7058,10 @@
         <v>247</v>
       </c>
       <c r="AA26" s="18" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
     </row>
-    <row r="27" spans="1:30" ht="135" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="17">
         <v>26</v>
       </c>
@@ -7075,7 +7117,7 @@
         <v>262</v>
       </c>
       <c r="V27" s="22" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="W27" s="16" t="s">
         <v>44</v>
@@ -7090,7 +7132,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="28" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="17">
         <v>27</v>
       </c>
@@ -7152,7 +7194,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="29" spans="1:30" ht="180" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="17">
         <v>28</v>
       </c>
@@ -7205,7 +7247,7 @@
         <v>278</v>
       </c>
       <c r="V29" s="22" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="W29" s="16" t="s">
         <v>44</v>
@@ -7220,7 +7262,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="30" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="17">
         <v>29</v>
       </c>
@@ -7279,7 +7321,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="31" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="17">
         <v>30</v>
       </c>
@@ -7329,7 +7371,7 @@
         <v>292</v>
       </c>
       <c r="V31" s="22" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="W31" s="16" t="s">
         <v>44</v>
@@ -7344,7 +7386,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="32" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="17">
         <v>31</v>
       </c>
@@ -7394,7 +7436,7 @@
         <v>251</v>
       </c>
       <c r="V32" s="22" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="W32" s="16" t="s">
         <v>44</v>
@@ -7406,13 +7448,13 @@
         <v>81</v>
       </c>
       <c r="Z32" s="14" t="s">
-        <v>968</v>
+        <v>961</v>
       </c>
       <c r="AC32" s="22" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
-    <row r="33" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="17">
         <v>32</v>
       </c>
@@ -7465,13 +7507,13 @@
         <v>81</v>
       </c>
       <c r="Z33" s="14" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="AC33" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="34" spans="1:30" ht="60" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="17">
         <v>33</v>
       </c>
@@ -7524,16 +7566,16 @@
         <v>81</v>
       </c>
       <c r="Z34" s="14" t="s">
-        <v>966</v>
+        <v>959</v>
       </c>
       <c r="AA34" s="18" t="s">
         <v>315</v>
       </c>
       <c r="AC34" s="22" t="s">
-        <v>967</v>
+        <v>960</v>
       </c>
     </row>
-    <row r="35" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="17">
         <v>34</v>
       </c>
@@ -7583,13 +7625,13 @@
         <v>81</v>
       </c>
       <c r="Z35" s="14" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="AC35" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="36" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="17">
         <v>35</v>
       </c>
@@ -7645,7 +7687,7 @@
         <v>331</v>
       </c>
       <c r="V36" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="W36" s="16" t="s">
         <v>44</v>
@@ -7654,16 +7696,16 @@
         <v>80</v>
       </c>
       <c r="Y36" s="24" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Z36" s="20" t="s">
         <v>332</v>
       </c>
       <c r="AC36" s="22" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
-    <row r="37" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="17">
         <v>36</v>
       </c>
@@ -7716,7 +7758,7 @@
         <v>331</v>
       </c>
       <c r="V37" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="W37" s="16" t="s">
         <v>44</v>
@@ -7725,16 +7767,16 @@
         <v>80</v>
       </c>
       <c r="Y37" s="24" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Z37" s="20" t="s">
         <v>340</v>
       </c>
       <c r="AC37" s="22" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
-    <row r="38" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="17">
         <v>37</v>
       </c>
@@ -7787,7 +7829,7 @@
         <v>351</v>
       </c>
       <c r="V38" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="W38" s="16" t="s">
         <v>44</v>
@@ -7796,16 +7838,16 @@
         <v>80</v>
       </c>
       <c r="Y38" s="24" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Z38" s="20" t="s">
         <v>352</v>
       </c>
       <c r="AC38" s="22" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="17">
         <v>38</v>
       </c>
@@ -7852,7 +7894,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="40" spans="1:30" ht="75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="17">
         <v>39</v>
       </c>
@@ -7878,7 +7920,7 @@
         <v>51</v>
       </c>
       <c r="V40" s="22" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="W40" s="16" t="s">
         <v>44</v>
@@ -7902,10 +7944,10 @@
         <v>365</v>
       </c>
       <c r="AD40" s="22" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
     </row>
-    <row r="41" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="17">
         <v>40</v>
       </c>
@@ -7958,16 +8000,16 @@
         <v>81</v>
       </c>
       <c r="Z41" s="14" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="AA41" s="18" t="s">
         <v>375</v>
       </c>
       <c r="AC41" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="42" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="17">
         <v>41</v>
       </c>
@@ -8020,13 +8062,13 @@
         <v>81</v>
       </c>
       <c r="Z42" s="14" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="AC42" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="43" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="17">
         <v>42</v>
       </c>
@@ -8079,13 +8121,13 @@
         <v>81</v>
       </c>
       <c r="Z43" s="14" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="AC43" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="44" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="17">
         <v>43</v>
       </c>
@@ -8138,13 +8180,13 @@
         <v>81</v>
       </c>
       <c r="Z44" s="14" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="AC44" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="17">
         <v>44</v>
       </c>
@@ -8182,7 +8224,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="46" spans="1:30" ht="90" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="17">
         <v>45</v>
       </c>
@@ -8247,16 +8289,16 @@
         <v>81</v>
       </c>
       <c r="Z46" s="14" t="s">
-        <v>962</v>
+        <v>955</v>
       </c>
       <c r="AA46" s="18" t="s">
         <v>409</v>
       </c>
       <c r="AC46" s="22" t="s">
-        <v>961</v>
+        <v>954</v>
       </c>
     </row>
-    <row r="47" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="17">
         <v>46</v>
       </c>
@@ -8309,13 +8351,13 @@
         <v>81</v>
       </c>
       <c r="Z47" s="14" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="AC47" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="48" spans="1:30" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="17">
         <v>47</v>
       </c>
@@ -8368,13 +8410,13 @@
         <v>81</v>
       </c>
       <c r="Z48" s="14" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="AC48" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="49" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="17">
         <v>48</v>
       </c>
@@ -8421,10 +8463,10 @@
         <v>428</v>
       </c>
       <c r="AC49" s="18" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
-    <row r="50" spans="1:31" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="17">
         <v>49</v>
       </c>
@@ -8468,10 +8510,10 @@
         <v>428</v>
       </c>
       <c r="AC50" s="18" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
-    <row r="51" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:31" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="17">
         <v>50</v>
       </c>
@@ -8518,10 +8560,10 @@
         <v>428</v>
       </c>
       <c r="AC51" s="18" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
-    <row r="52" spans="1:31" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="17">
         <v>51</v>
       </c>
@@ -8568,10 +8610,10 @@
         <v>428</v>
       </c>
       <c r="AC52" s="18" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
-    <row r="53" spans="1:31" ht="150" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="17">
         <v>52</v>
       </c>
@@ -8594,13 +8636,13 @@
         <v>443</v>
       </c>
       <c r="M53" s="35" t="s">
-        <v>993</v>
+        <v>986</v>
       </c>
       <c r="N53" s="35" t="s">
-        <v>995</v>
+        <v>988</v>
       </c>
       <c r="V53" s="35" t="s">
-        <v>996</v>
+        <v>989</v>
       </c>
       <c r="W53" s="24" t="s">
         <v>44</v>
@@ -8612,16 +8654,16 @@
         <v>302</v>
       </c>
       <c r="Z53" s="14" t="s">
-        <v>994</v>
+        <v>987</v>
       </c>
       <c r="AC53" s="22" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="AE53" s="35" t="s">
-        <v>999</v>
+        <v>992</v>
       </c>
     </row>
-    <row r="54" spans="1:31" ht="180" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="17">
         <v>53</v>
       </c>
@@ -8668,7 +8710,7 @@
         <v>453</v>
       </c>
       <c r="V54" s="22" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="W54" s="16" t="s">
         <v>44</v>
@@ -8689,7 +8731,7 @@
         <v>456</v>
       </c>
       <c r="AC54" s="22" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="AD54" s="18" t="s">
         <v>457</v>
@@ -8698,7 +8740,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="55" spans="1:31" ht="90" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:31" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="17">
         <v>54</v>
       </c>
@@ -8721,19 +8763,19 @@
         <v>461</v>
       </c>
       <c r="M55" s="22" t="s">
+        <v>813</v>
+      </c>
+      <c r="N55" s="22" t="s">
         <v>814</v>
       </c>
-      <c r="N55" s="22" t="s">
+      <c r="P55" s="24" t="s">
+        <v>876</v>
+      </c>
+      <c r="T55" s="22" t="s">
         <v>815</v>
       </c>
-      <c r="P55" s="24" t="s">
+      <c r="V55" s="27" t="s">
         <v>877</v>
-      </c>
-      <c r="T55" s="22" t="s">
-        <v>816</v>
-      </c>
-      <c r="V55" s="27" t="s">
-        <v>878</v>
       </c>
       <c r="W55" s="24" t="s">
         <v>44</v>
@@ -8745,13 +8787,13 @@
         <v>92</v>
       </c>
       <c r="Z55" s="14" t="s">
-        <v>880</v>
-      </c>
-      <c r="AC55" s="27" t="s">
-        <v>941</v>
+        <v>879</v>
+      </c>
+      <c r="AC55" s="36" t="s">
+        <v>936</v>
       </c>
     </row>
-    <row r="56" spans="1:31" ht="120" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="17">
         <v>55</v>
       </c>
@@ -8798,7 +8840,7 @@
         <v>471</v>
       </c>
       <c r="V56" s="22" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="W56" s="16" t="s">
         <v>44</v>
@@ -8813,7 +8855,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="57" spans="1:31" ht="90" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="17">
         <v>56</v>
       </c>
@@ -8857,7 +8899,7 @@
         <v>471</v>
       </c>
       <c r="V57" s="22" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="W57" s="16" t="s">
         <v>44</v>
@@ -8869,10 +8911,10 @@
         <v>92</v>
       </c>
       <c r="Z57" s="14" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
     </row>
-    <row r="58" spans="1:31" ht="75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="17">
         <v>57</v>
       </c>
@@ -8919,7 +8961,7 @@
         <v>483</v>
       </c>
       <c r="V58" s="22" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="W58" s="16" t="s">
         <v>44</v>
@@ -8931,16 +8973,16 @@
         <v>81</v>
       </c>
       <c r="Z58" s="22" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="AA58" s="18" t="s">
         <v>455</v>
       </c>
       <c r="AC58" s="18" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
     </row>
-    <row r="59" spans="1:31" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:31" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="17">
         <v>58</v>
       </c>
@@ -8990,10 +9032,10 @@
         <v>81</v>
       </c>
       <c r="Z59" s="20" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
     </row>
-    <row r="60" spans="1:31" ht="195" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="17">
         <v>59</v>
       </c>
@@ -9049,7 +9091,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="61" spans="1:31" ht="195" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="17">
         <v>60</v>
       </c>
@@ -9079,7 +9121,7 @@
       </c>
       <c r="T61" s="21"/>
       <c r="V61" s="22" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="W61" s="16" t="s">
         <v>147</v>
@@ -9100,10 +9142,10 @@
         <v>504</v>
       </c>
       <c r="AC61" s="22" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="AD61" s="23" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
     </row>
     <row r="62" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
@@ -9150,7 +9192,7 @@
         <v>513</v>
       </c>
       <c r="V62" s="22" t="s">
-        <v>963</v>
+        <v>956</v>
       </c>
       <c r="W62" s="16" t="s">
         <v>44</v>
@@ -9165,10 +9207,10 @@
         <v>514</v>
       </c>
       <c r="AC62" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="63" spans="1:31" ht="135" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="17">
         <v>62</v>
       </c>
@@ -9209,7 +9251,7 @@
         <v>520</v>
       </c>
       <c r="V63" s="22" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="W63" s="16" t="s">
         <v>44</v>
@@ -9224,7 +9266,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="64" spans="1:31" ht="135" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="17">
         <v>63</v>
       </c>
@@ -9265,7 +9307,7 @@
         <v>520</v>
       </c>
       <c r="V64" s="22" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="W64" s="16" t="s">
         <v>44</v>
@@ -9280,7 +9322,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="65" spans="1:31" ht="165" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="17">
         <v>64</v>
       </c>
@@ -9362,7 +9404,7 @@
         <v>520</v>
       </c>
       <c r="V66" s="22" t="s">
-        <v>964</v>
+        <v>957</v>
       </c>
       <c r="W66" s="16" t="s">
         <v>44</v>
@@ -9377,7 +9419,7 @@
         <v>538</v>
       </c>
       <c r="AC66" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
     <row r="67" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
@@ -9424,7 +9466,7 @@
         <v>513</v>
       </c>
       <c r="V67" s="22" t="s">
-        <v>965</v>
+        <v>958</v>
       </c>
       <c r="W67" s="16" t="s">
         <v>44</v>
@@ -9436,13 +9478,13 @@
         <v>81</v>
       </c>
       <c r="Z67" s="20" t="s">
-        <v>546</v>
+        <v>1003</v>
       </c>
       <c r="AC67" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="68" spans="1:31" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:31" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="17">
         <v>67</v>
       </c>
@@ -9450,13 +9492,13 @@
         <v>33</v>
       </c>
       <c r="C68" s="7" t="s">
+        <v>546</v>
+      </c>
+      <c r="D68" s="16" t="s">
         <v>547</v>
       </c>
-      <c r="D68" s="16" t="s">
-        <v>548</v>
-      </c>
       <c r="E68" s="16" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F68" s="7" t="s">
         <v>205</v>
@@ -9483,13 +9525,13 @@
         <v>147</v>
       </c>
       <c r="AB68" s="22" t="s">
+        <v>884</v>
+      </c>
+      <c r="AD68" s="23" t="s">
         <v>885</v>
       </c>
-      <c r="AD68" s="23" t="s">
-        <v>886</v>
-      </c>
     </row>
-    <row r="69" spans="1:31" ht="90" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:31" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="17">
         <v>68</v>
       </c>
@@ -9497,19 +9539,19 @@
         <v>33</v>
       </c>
       <c r="C69" s="7" t="s">
+        <v>548</v>
+      </c>
+      <c r="D69" s="16" t="s">
         <v>549</v>
       </c>
-      <c r="D69" s="16" t="s">
+      <c r="E69" s="16" t="s">
         <v>550</v>
-      </c>
-      <c r="E69" s="16" t="s">
-        <v>551</v>
       </c>
       <c r="F69" s="7" t="s">
         <v>63</v>
       </c>
       <c r="L69" s="12" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="M69" s="18" t="s">
         <v>51</v>
@@ -9527,13 +9569,13 @@
         <v>147</v>
       </c>
       <c r="AB69" s="22" t="s">
+        <v>884</v>
+      </c>
+      <c r="AD69" s="23" t="s">
         <v>885</v>
       </c>
-      <c r="AD69" s="23" t="s">
-        <v>886</v>
-      </c>
     </row>
-    <row r="70" spans="1:31" ht="180" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" ht="180" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="17">
         <v>69</v>
       </c>
@@ -9541,43 +9583,43 @@
         <v>33</v>
       </c>
       <c r="C70" s="7" t="s">
+        <v>552</v>
+      </c>
+      <c r="D70" s="16" t="s">
         <v>553</v>
       </c>
-      <c r="D70" s="16" t="s">
+      <c r="E70" s="16" t="s">
         <v>554</v>
-      </c>
-      <c r="E70" s="16" t="s">
-        <v>555</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K70" s="7" t="s">
+        <v>555</v>
+      </c>
+      <c r="L70" s="12" t="s">
         <v>556</v>
       </c>
-      <c r="L70" s="12" t="s">
+      <c r="M70" s="18" t="s">
         <v>557</v>
       </c>
-      <c r="M70" s="18" t="s">
+      <c r="N70" s="18" t="s">
         <v>558</v>
       </c>
-      <c r="N70" s="18" t="s">
+      <c r="O70" s="16" t="s">
         <v>559</v>
       </c>
-      <c r="O70" s="16" t="s">
+      <c r="P70" s="16" t="s">
         <v>560</v>
-      </c>
-      <c r="P70" s="16" t="s">
-        <v>561</v>
       </c>
       <c r="S70" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T70" s="18" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="V70" s="22" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="W70" s="16" t="s">
         <v>44</v>
@@ -9589,13 +9631,13 @@
         <v>92</v>
       </c>
       <c r="Z70" s="20" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="AC70" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="71" spans="1:31" ht="105" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:31" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="17">
         <v>70</v>
       </c>
@@ -9603,40 +9645,40 @@
         <v>33</v>
       </c>
       <c r="C71" s="7" t="s">
+        <v>563</v>
+      </c>
+      <c r="D71" s="16" t="s">
         <v>564</v>
       </c>
-      <c r="D71" s="16" t="s">
+      <c r="E71" s="16" t="s">
         <v>565</v>
-      </c>
-      <c r="E71" s="16" t="s">
-        <v>566</v>
       </c>
       <c r="F71" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K71" s="7" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="L71" s="12" t="s">
+        <v>566</v>
+      </c>
+      <c r="M71" s="18" t="s">
         <v>567</v>
       </c>
-      <c r="M71" s="18" t="s">
+      <c r="N71" s="18" t="s">
         <v>568</v>
       </c>
-      <c r="N71" s="18" t="s">
+      <c r="O71" s="16" t="s">
         <v>569</v>
       </c>
-      <c r="O71" s="16" t="s">
+      <c r="P71" s="16" t="s">
         <v>570</v>
-      </c>
-      <c r="P71" s="16" t="s">
-        <v>571</v>
       </c>
       <c r="S71" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T71" s="21" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="W71" s="16" t="s">
         <v>44</v>
@@ -9648,13 +9690,13 @@
         <v>92</v>
       </c>
       <c r="Z71" s="20" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="AC71" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="72" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:31" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="17">
         <v>71</v>
       </c>
@@ -9662,46 +9704,46 @@
         <v>33</v>
       </c>
       <c r="C72" s="7" t="s">
+        <v>573</v>
+      </c>
+      <c r="D72" s="16" t="s">
         <v>574</v>
       </c>
-      <c r="D72" s="16" t="s">
+      <c r="E72" s="16" t="s">
         <v>575</v>
-      </c>
-      <c r="E72" s="16" t="s">
-        <v>576</v>
       </c>
       <c r="F72" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J72" s="7" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="K72" s="7" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="L72" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M72" s="18" t="s">
+        <v>577</v>
+      </c>
+      <c r="N72" s="18" t="s">
         <v>578</v>
       </c>
-      <c r="N72" s="18" t="s">
+      <c r="O72" s="16" t="s">
+        <v>559</v>
+      </c>
+      <c r="P72" s="16" t="s">
         <v>579</v>
-      </c>
-      <c r="O72" s="16" t="s">
-        <v>560</v>
-      </c>
-      <c r="P72" s="16" t="s">
-        <v>580</v>
       </c>
       <c r="S72" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T72" s="18" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="V72" s="22" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="W72" s="16" t="s">
         <v>44</v>
@@ -9713,13 +9755,13 @@
         <v>81</v>
       </c>
       <c r="Z72" s="20" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="AC72" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="73" spans="1:31" ht="135" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:31" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="17">
         <v>72</v>
       </c>
@@ -9727,43 +9769,43 @@
         <v>33</v>
       </c>
       <c r="C73" s="7" t="s">
+        <v>581</v>
+      </c>
+      <c r="D73" s="16" t="s">
         <v>582</v>
       </c>
-      <c r="D73" s="16" t="s">
+      <c r="E73" s="16" t="s">
         <v>583</v>
-      </c>
-      <c r="E73" s="16" t="s">
-        <v>584</v>
       </c>
       <c r="F73" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J73" s="7" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="L73" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M73" s="18" t="s">
+        <v>585</v>
+      </c>
+      <c r="N73" s="18" t="s">
         <v>586</v>
       </c>
-      <c r="N73" s="18" t="s">
+      <c r="O73" s="16" t="s">
         <v>587</v>
       </c>
-      <c r="O73" s="16" t="s">
+      <c r="P73" s="16" t="s">
         <v>588</v>
-      </c>
-      <c r="P73" s="16" t="s">
-        <v>589</v>
       </c>
       <c r="S73" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T73" s="18" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="V73" s="27" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="W73" s="16" t="s">
         <v>44</v>
@@ -9775,13 +9817,13 @@
         <v>81</v>
       </c>
       <c r="Z73" s="20" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="AC73" s="27" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
     </row>
-    <row r="74" spans="1:31" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="17">
         <v>73</v>
       </c>
@@ -9789,46 +9831,46 @@
         <v>33</v>
       </c>
       <c r="C74" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="D74" s="16" t="s">
         <v>592</v>
       </c>
-      <c r="D74" s="16" t="s">
+      <c r="E74" s="16" t="s">
         <v>593</v>
-      </c>
-      <c r="E74" s="16" t="s">
-        <v>594</v>
       </c>
       <c r="F74" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J74" s="7" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="K74" s="7" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="L74" s="12" t="s">
         <v>121</v>
       </c>
       <c r="M74" s="18" t="s">
+        <v>595</v>
+      </c>
+      <c r="N74" s="18" t="s">
         <v>596</v>
       </c>
-      <c r="N74" s="18" t="s">
-        <v>597</v>
-      </c>
       <c r="O74" s="16" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="P74" s="16" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="S74" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T74" s="18" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="V74" s="22" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="W74" s="16" t="s">
         <v>44</v>
@@ -9840,13 +9882,13 @@
         <v>81</v>
       </c>
       <c r="Z74" s="20" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="AC74" s="22" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
     </row>
-    <row r="75" spans="1:31" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" ht="285" x14ac:dyDescent="0.25">
       <c r="A75" s="17">
         <v>74</v>
       </c>
@@ -9854,31 +9896,31 @@
         <v>33</v>
       </c>
       <c r="C75" s="7" t="s">
+        <v>598</v>
+      </c>
+      <c r="D75" s="16" t="s">
         <v>599</v>
       </c>
-      <c r="D75" s="16" t="s">
+      <c r="E75" s="16" t="s">
         <v>600</v>
-      </c>
-      <c r="E75" s="16" t="s">
-        <v>601</v>
       </c>
       <c r="F75" s="7" t="s">
         <v>205</v>
       </c>
       <c r="J75" s="7" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="M75" s="22" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="N75" s="22" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="O75" s="24" t="s">
+        <v>604</v>
+      </c>
+      <c r="P75" s="24" t="s">
         <v>605</v>
-      </c>
-      <c r="P75" s="24" t="s">
-        <v>606</v>
       </c>
       <c r="Q75" s="24"/>
       <c r="R75" s="24"/>
@@ -9886,7 +9928,7 @@
         <v>43</v>
       </c>
       <c r="T75" s="33" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="W75" s="32" t="s">
         <v>44</v>
@@ -9898,13 +9940,13 @@
         <v>81</v>
       </c>
       <c r="Z75" s="14" t="s">
-        <v>950</v>
+        <v>1004</v>
       </c>
       <c r="AA75" s="22" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="AC75" s="22" t="s">
-        <v>948</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="76" spans="1:31" ht="225" x14ac:dyDescent="0.25">
@@ -9915,37 +9957,37 @@
         <v>33</v>
       </c>
       <c r="C76" s="7" t="s">
+        <v>608</v>
+      </c>
+      <c r="D76" s="16" t="s">
         <v>609</v>
       </c>
-      <c r="D76" s="16" t="s">
+      <c r="E76" s="16" t="s">
         <v>610</v>
-      </c>
-      <c r="E76" s="16" t="s">
-        <v>611</v>
       </c>
       <c r="F76" s="7" t="s">
         <v>63</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="M76" s="18" t="s">
+        <v>602</v>
+      </c>
+      <c r="N76" s="18" t="s">
         <v>603</v>
       </c>
-      <c r="N76" s="18" t="s">
+      <c r="O76" s="16" t="s">
         <v>604</v>
       </c>
-      <c r="O76" s="16" t="s">
+      <c r="P76" s="16" t="s">
         <v>605</v>
-      </c>
-      <c r="P76" s="16" t="s">
-        <v>606</v>
       </c>
       <c r="S76" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T76" s="18" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="W76" s="16" t="s">
         <v>44</v>
@@ -9954,16 +9996,16 @@
         <v>80</v>
       </c>
       <c r="Y76" s="24" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="Z76" s="20" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AC76" s="22" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
-    <row r="77" spans="1:31" ht="105" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="17">
         <v>76</v>
       </c>
@@ -9971,40 +10013,40 @@
         <v>33</v>
       </c>
       <c r="C77" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="D77" s="16" t="s">
         <v>614</v>
       </c>
-      <c r="D77" s="16" t="s">
-        <v>615</v>
-      </c>
       <c r="E77" s="16" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="F77" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K77" s="7" t="s">
+        <v>615</v>
+      </c>
+      <c r="L77" s="12" t="s">
         <v>616</v>
       </c>
-      <c r="L77" s="12" t="s">
+      <c r="M77" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="M77" s="18" t="s">
+      <c r="N77" s="18" t="s">
         <v>618</v>
       </c>
-      <c r="N77" s="18" t="s">
+      <c r="O77" s="16" t="s">
+        <v>604</v>
+      </c>
+      <c r="P77" s="16" t="s">
         <v>619</v>
-      </c>
-      <c r="O77" s="16" t="s">
-        <v>605</v>
-      </c>
-      <c r="P77" s="16" t="s">
-        <v>620</v>
       </c>
       <c r="S77" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T77" s="18" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="W77" s="16" t="s">
         <v>44</v>
@@ -10016,10 +10058,10 @@
         <v>92</v>
       </c>
       <c r="Z77" s="28" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
-    <row r="78" spans="1:31" ht="135" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="17">
         <v>77</v>
       </c>
@@ -10027,37 +10069,37 @@
         <v>33</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="D78" s="16" t="s">
         <v>623</v>
       </c>
-      <c r="D78" s="16" t="s">
+      <c r="E78" s="16" t="s">
         <v>624</v>
-      </c>
-      <c r="E78" s="16" t="s">
-        <v>625</v>
       </c>
       <c r="F78" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J78" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="K78" s="7" t="s">
         <v>626</v>
       </c>
-      <c r="K78" s="7" t="s">
+      <c r="L78" s="12" t="s">
         <v>627</v>
       </c>
-      <c r="L78" s="12" t="s">
+      <c r="M78" s="22" t="s">
+        <v>892</v>
+      </c>
+      <c r="N78" s="22" t="s">
+        <v>891</v>
+      </c>
+      <c r="O78" s="24" t="s">
         <v>628</v>
       </c>
-      <c r="M78" s="22" t="s">
-        <v>893</v>
-      </c>
-      <c r="N78" s="22" t="s">
-        <v>892</v>
-      </c>
-      <c r="O78" s="24" t="s">
+      <c r="P78" s="24" t="s">
         <v>629</v>
-      </c>
-      <c r="P78" s="24" t="s">
-        <v>630</v>
       </c>
       <c r="Q78" s="24"/>
       <c r="R78" s="24"/>
@@ -10065,10 +10107,10 @@
         <v>43</v>
       </c>
       <c r="T78" s="31" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="V78" s="35" t="s">
-        <v>998</v>
+        <v>991</v>
       </c>
       <c r="W78" s="16" t="s">
         <v>44</v>
@@ -10080,16 +10122,16 @@
         <v>81</v>
       </c>
       <c r="Z78" s="34" t="s">
-        <v>997</v>
+        <v>990</v>
       </c>
       <c r="AC78" s="22" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="AE78" s="35" t="s">
-        <v>1000</v>
+        <v>993</v>
       </c>
     </row>
-    <row r="79" spans="1:31" ht="90" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="17">
         <v>78</v>
       </c>
@@ -10097,37 +10139,37 @@
         <v>33</v>
       </c>
       <c r="C79" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="D79" s="16" t="s">
         <v>632</v>
       </c>
-      <c r="D79" s="16" t="s">
+      <c r="E79" s="16" t="s">
         <v>633</v>
-      </c>
-      <c r="E79" s="16" t="s">
-        <v>634</v>
       </c>
       <c r="F79" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I79" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="J79" s="7" t="s">
         <v>635</v>
       </c>
-      <c r="J79" s="7" t="s">
-        <v>636</v>
-      </c>
       <c r="L79" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M79" s="22" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
       <c r="N79" s="22" t="s">
-        <v>951</v>
+        <v>944</v>
       </c>
       <c r="T79" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V79" s="22" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="W79" s="24" t="s">
         <v>44</v>
@@ -10139,16 +10181,16 @@
         <v>81</v>
       </c>
       <c r="Z79" s="14" t="s">
-        <v>970</v>
+        <v>963</v>
       </c>
       <c r="AB79" s="22" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="AD79" s="23" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
-    <row r="80" spans="1:31" ht="90" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:31" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="17">
         <v>79</v>
       </c>
@@ -10156,37 +10198,37 @@
         <v>33</v>
       </c>
       <c r="C80" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="D80" s="16" t="s">
         <v>637</v>
       </c>
-      <c r="D80" s="16" t="s">
+      <c r="E80" s="16" t="s">
         <v>638</v>
-      </c>
-      <c r="E80" s="16" t="s">
-        <v>639</v>
       </c>
       <c r="F80" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I80" s="7" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="J80" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L80" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M80" s="22" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
       <c r="N80" s="22" t="s">
-        <v>952</v>
+        <v>945</v>
       </c>
       <c r="T80" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V80" s="22" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="W80" s="24" t="s">
         <v>44</v>
@@ -10198,19 +10240,19 @@
         <v>81</v>
       </c>
       <c r="Z80" s="14" t="s">
-        <v>971</v>
+        <v>964</v>
       </c>
       <c r="AB80" s="22" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="AC80" s="22" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
       <c r="AD80" s="23" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
-    <row r="81" spans="1:33" ht="135" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:33" ht="135" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="17">
         <v>80</v>
       </c>
@@ -10218,37 +10260,37 @@
         <v>33</v>
       </c>
       <c r="C81" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="D81" s="16" t="s">
         <v>641</v>
       </c>
-      <c r="D81" s="16" t="s">
+      <c r="E81" s="16" t="s">
         <v>642</v>
-      </c>
-      <c r="E81" s="16" t="s">
-        <v>643</v>
       </c>
       <c r="F81" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I81" s="7" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="J81" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L81" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M81" s="22" t="s">
-        <v>958</v>
+        <v>951</v>
       </c>
       <c r="N81" s="22" t="s">
-        <v>955</v>
+        <v>948</v>
       </c>
       <c r="T81" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V81" s="22" t="s">
-        <v>989</v>
+        <v>982</v>
       </c>
       <c r="W81" s="24" t="s">
         <v>44</v>
@@ -10260,19 +10302,19 @@
         <v>81</v>
       </c>
       <c r="Z81" s="14" t="s">
-        <v>972</v>
+        <v>965</v>
       </c>
       <c r="AB81" s="22" t="s">
+        <v>889</v>
+      </c>
+      <c r="AC81" s="27" t="s">
         <v>890</v>
       </c>
-      <c r="AC81" s="27" t="s">
-        <v>891</v>
-      </c>
       <c r="AD81" s="23" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
-    <row r="82" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="17">
         <v>81</v>
       </c>
@@ -10280,46 +10322,46 @@
         <v>33</v>
       </c>
       <c r="C82" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="D82" s="16" t="s">
         <v>645</v>
       </c>
-      <c r="D82" s="16" t="s">
+      <c r="E82" s="16" t="s">
         <v>646</v>
-      </c>
-      <c r="E82" s="16" t="s">
-        <v>647</v>
       </c>
       <c r="F82" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I82" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="J82" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="L82" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="M82" s="18" t="s">
         <v>648</v>
       </c>
-      <c r="J82" s="7" t="s">
-        <v>636</v>
-      </c>
-      <c r="L82" s="12" t="s">
+      <c r="N82" s="18" t="s">
+        <v>649</v>
+      </c>
+      <c r="O82" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="M82" s="18" t="s">
-        <v>649</v>
-      </c>
-      <c r="N82" s="18" t="s">
+      <c r="P82" s="16" t="s">
         <v>650</v>
-      </c>
-      <c r="O82" s="16" t="s">
-        <v>629</v>
-      </c>
-      <c r="P82" s="16" t="s">
-        <v>651</v>
       </c>
       <c r="S82" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T82" s="18" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="V82" s="22" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="W82" s="16" t="s">
         <v>44</v>
@@ -10331,19 +10373,19 @@
         <v>92</v>
       </c>
       <c r="Z82" s="14" t="s">
-        <v>973</v>
+        <v>966</v>
       </c>
       <c r="AB82" s="22" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="AC82" s="22" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
       <c r="AD82" s="23" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
-    <row r="83" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="17">
         <v>82</v>
       </c>
@@ -10351,37 +10393,37 @@
         <v>33</v>
       </c>
       <c r="C83" s="7" t="s">
+        <v>653</v>
+      </c>
+      <c r="D83" s="16" t="s">
         <v>654</v>
       </c>
-      <c r="D83" s="16" t="s">
+      <c r="E83" s="16" t="s">
         <v>655</v>
-      </c>
-      <c r="E83" s="16" t="s">
-        <v>656</v>
       </c>
       <c r="F83" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I83" s="7" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="J83" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L83" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M83" s="22" t="s">
-        <v>959</v>
+        <v>952</v>
       </c>
       <c r="N83" s="22" t="s">
-        <v>953</v>
+        <v>946</v>
       </c>
       <c r="T83" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V83" s="22" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="W83" s="24" t="s">
         <v>44</v>
@@ -10393,19 +10435,19 @@
         <v>81</v>
       </c>
       <c r="Z83" s="14" t="s">
-        <v>974</v>
+        <v>967</v>
       </c>
       <c r="AB83" s="22" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="AC83" s="22" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
       <c r="AD83" s="23" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
     </row>
-    <row r="84" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:33" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="17">
         <v>83</v>
       </c>
@@ -10413,25 +10455,25 @@
         <v>33</v>
       </c>
       <c r="C84" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="D84" s="16" t="s">
         <v>658</v>
       </c>
-      <c r="D84" s="16" t="s">
+      <c r="E84" s="16" t="s">
         <v>659</v>
-      </c>
-      <c r="E84" s="16" t="s">
-        <v>660</v>
       </c>
       <c r="F84" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I84" s="7" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="J84" s="7" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="L84" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M84" s="18" t="s">
         <v>51</v>
@@ -10449,16 +10491,16 @@
         <v>147</v>
       </c>
       <c r="AB84" s="22" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="AC84" s="22" t="s">
-        <v>954</v>
+        <v>947</v>
       </c>
       <c r="AD84" s="23" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
-    <row r="85" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="17">
         <v>84</v>
       </c>
@@ -10466,49 +10508,49 @@
         <v>33</v>
       </c>
       <c r="C85" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="D85" s="16" t="s">
         <v>662</v>
       </c>
-      <c r="D85" s="16" t="s">
+      <c r="E85" s="16" t="s">
         <v>663</v>
-      </c>
-      <c r="E85" s="16" t="s">
-        <v>664</v>
       </c>
       <c r="F85" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I85" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="J85" s="7" t="s">
         <v>665</v>
       </c>
-      <c r="J85" s="7" t="s">
+      <c r="K85" s="7" t="s">
         <v>666</v>
       </c>
-      <c r="K85" s="7" t="s">
+      <c r="L85" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="M85" s="18" t="s">
         <v>667</v>
       </c>
-      <c r="L85" s="12" t="s">
+      <c r="N85" s="18" t="s">
+        <v>668</v>
+      </c>
+      <c r="O85" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="M85" s="18" t="s">
-        <v>668</v>
-      </c>
-      <c r="N85" s="18" t="s">
-        <v>669</v>
-      </c>
-      <c r="O85" s="16" t="s">
+      <c r="P85" s="16" t="s">
         <v>629</v>
-      </c>
-      <c r="P85" s="16" t="s">
-        <v>630</v>
       </c>
       <c r="S85" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T85" s="18" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="V85" s="22" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="W85" s="16" t="s">
         <v>44</v>
@@ -10520,13 +10562,13 @@
         <v>92</v>
       </c>
       <c r="Z85" s="14" t="s">
-        <v>973</v>
+        <v>966</v>
       </c>
       <c r="AB85" s="22" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
     </row>
-    <row r="86" spans="1:33" ht="375" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:33" ht="330" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="17">
         <v>85</v>
       </c>
@@ -10534,13 +10576,13 @@
         <v>33</v>
       </c>
       <c r="C86" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="D86" s="19" t="s">
         <v>670</v>
       </c>
-      <c r="D86" s="19" t="s">
+      <c r="E86" s="19" t="s">
         <v>671</v>
-      </c>
-      <c r="E86" s="19" t="s">
-        <v>672</v>
       </c>
       <c r="F86" s="13" t="s">
         <v>63</v>
@@ -10548,36 +10590,36 @@
       <c r="G86" s="13"/>
       <c r="H86" s="13"/>
       <c r="I86" s="13" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="J86" s="13" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="K86" s="13"/>
       <c r="L86" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M86" s="28" t="s">
+        <v>673</v>
+      </c>
+      <c r="N86" s="22" t="s">
+        <v>668</v>
+      </c>
+      <c r="O86" s="19" t="s">
         <v>674</v>
       </c>
-      <c r="N86" s="22" t="s">
-        <v>669</v>
-      </c>
-      <c r="O86" s="19" t="s">
+      <c r="P86" s="19" t="s">
         <v>675</v>
-      </c>
-      <c r="P86" s="19" t="s">
-        <v>676</v>
       </c>
       <c r="Q86" s="19"/>
       <c r="R86" s="30" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="S86" s="19" t="s">
         <v>43</v>
       </c>
       <c r="T86" s="29" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="U86" s="19"/>
       <c r="V86" s="28"/>
@@ -10591,21 +10633,21 @@
         <v>81</v>
       </c>
       <c r="Z86" s="14" t="s">
-        <v>895</v>
+        <v>1000</v>
       </c>
       <c r="AA86" s="28" t="s">
         <v>455</v>
       </c>
       <c r="AB86" s="28"/>
       <c r="AC86" s="14" t="s">
-        <v>896</v>
+        <v>1001</v>
       </c>
       <c r="AD86" s="28"/>
       <c r="AE86" s="28"/>
       <c r="AF86" s="19"/>
       <c r="AG86" s="19"/>
     </row>
-    <row r="87" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="17">
         <v>86</v>
       </c>
@@ -10613,37 +10655,37 @@
         <v>33</v>
       </c>
       <c r="C87" s="7" t="s">
+        <v>678</v>
+      </c>
+      <c r="D87" s="16" t="s">
         <v>679</v>
       </c>
-      <c r="D87" s="16" t="s">
+      <c r="E87" s="16" t="s">
         <v>680</v>
-      </c>
-      <c r="E87" s="16" t="s">
-        <v>681</v>
       </c>
       <c r="F87" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I87" s="7" t="s">
+        <v>681</v>
+      </c>
+      <c r="J87" s="7" t="s">
         <v>682</v>
       </c>
-      <c r="J87" s="7" t="s">
-        <v>683</v>
-      </c>
       <c r="L87" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M87" s="22" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="N87" s="22" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="T87" s="22" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="V87" s="22" t="s">
-        <v>991</v>
+        <v>984</v>
       </c>
       <c r="W87" s="24" t="s">
         <v>44</v>
@@ -10655,14 +10697,14 @@
         <v>81</v>
       </c>
       <c r="Z87" s="14" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="AB87" s="28"/>
       <c r="AC87" s="22" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
     </row>
-    <row r="88" spans="1:33" ht="60" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:33" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="17">
         <v>87</v>
       </c>
@@ -10670,46 +10712,46 @@
         <v>33</v>
       </c>
       <c r="C88" s="7" t="s">
+        <v>683</v>
+      </c>
+      <c r="D88" s="16" t="s">
         <v>684</v>
       </c>
-      <c r="D88" s="16" t="s">
+      <c r="E88" s="16" t="s">
         <v>685</v>
-      </c>
-      <c r="E88" s="16" t="s">
-        <v>686</v>
       </c>
       <c r="F88" s="7" t="s">
         <v>63</v>
       </c>
       <c r="I88" s="7" t="s">
+        <v>686</v>
+      </c>
+      <c r="J88" s="7" t="s">
+        <v>682</v>
+      </c>
+      <c r="K88" s="7" t="s">
         <v>687</v>
       </c>
-      <c r="J88" s="7" t="s">
-        <v>683</v>
-      </c>
-      <c r="K88" s="7" t="s">
+      <c r="L88" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="M88" s="18" t="s">
         <v>688</v>
       </c>
-      <c r="L88" s="12" t="s">
+      <c r="N88" s="18" t="s">
+        <v>689</v>
+      </c>
+      <c r="O88" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="M88" s="18" t="s">
-        <v>689</v>
-      </c>
-      <c r="N88" s="18" t="s">
+      <c r="P88" s="16" t="s">
         <v>690</v>
-      </c>
-      <c r="O88" s="16" t="s">
-        <v>629</v>
-      </c>
-      <c r="P88" s="16" t="s">
-        <v>691</v>
       </c>
       <c r="S88" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T88" s="21" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="W88" s="16" t="s">
         <v>44</v>
@@ -10721,10 +10763,10 @@
         <v>92</v>
       </c>
       <c r="Z88" s="20" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
-    <row r="89" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:33" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="17">
         <v>88</v>
       </c>
@@ -10732,22 +10774,22 @@
         <v>33</v>
       </c>
       <c r="C89" s="7" t="s">
+        <v>691</v>
+      </c>
+      <c r="D89" s="16" t="s">
         <v>692</v>
       </c>
-      <c r="D89" s="16" t="s">
-        <v>693</v>
-      </c>
       <c r="E89" s="16" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F89" s="7" t="s">
         <v>63</v>
       </c>
       <c r="K89" s="7" t="s">
+        <v>693</v>
+      </c>
+      <c r="L89" s="12" t="s">
         <v>694</v>
-      </c>
-      <c r="L89" s="12" t="s">
-        <v>695</v>
       </c>
       <c r="M89" s="18" t="s">
         <v>51</v>
@@ -10765,7 +10807,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="90" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="17">
         <v>89</v>
       </c>
@@ -10773,46 +10815,46 @@
         <v>33</v>
       </c>
       <c r="C90" s="7" t="s">
+        <v>695</v>
+      </c>
+      <c r="D90" s="16" t="s">
         <v>696</v>
       </c>
-      <c r="D90" s="16" t="s">
+      <c r="E90" s="16" t="s">
         <v>697</v>
-      </c>
-      <c r="E90" s="16" t="s">
-        <v>698</v>
       </c>
       <c r="F90" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J90" s="7" t="s">
+        <v>698</v>
+      </c>
+      <c r="K90" s="7" t="s">
         <v>699</v>
       </c>
-      <c r="K90" s="7" t="s">
+      <c r="L90" s="12" t="s">
+        <v>627</v>
+      </c>
+      <c r="M90" s="18" t="s">
         <v>700</v>
       </c>
-      <c r="L90" s="12" t="s">
+      <c r="N90" s="18" t="s">
+        <v>701</v>
+      </c>
+      <c r="O90" s="16" t="s">
         <v>628</v>
       </c>
-      <c r="M90" s="18" t="s">
-        <v>701</v>
-      </c>
-      <c r="N90" s="18" t="s">
+      <c r="P90" s="16" t="s">
         <v>702</v>
-      </c>
-      <c r="O90" s="16" t="s">
-        <v>629</v>
-      </c>
-      <c r="P90" s="16" t="s">
-        <v>703</v>
       </c>
       <c r="S90" s="16" t="s">
         <v>43</v>
       </c>
       <c r="T90" s="18" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="V90" s="22" t="s">
-        <v>990</v>
+        <v>983</v>
       </c>
       <c r="W90" s="16" t="s">
         <v>44</v>
@@ -10824,16 +10866,16 @@
         <v>92</v>
       </c>
       <c r="Z90" s="14" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="AA90" s="18" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="AC90" s="22" t="s">
-        <v>969</v>
+        <v>962</v>
       </c>
     </row>
-    <row r="91" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="17">
         <v>90</v>
       </c>
@@ -10841,34 +10883,34 @@
         <v>33</v>
       </c>
       <c r="C91" s="7" t="s">
+        <v>704</v>
+      </c>
+      <c r="D91" s="16" t="s">
         <v>705</v>
       </c>
-      <c r="D91" s="16" t="s">
+      <c r="E91" s="16" t="s">
         <v>706</v>
-      </c>
-      <c r="E91" s="16" t="s">
-        <v>707</v>
       </c>
       <c r="F91" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J91" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L91" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M91" s="22" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="N91" s="22" t="s">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="T91" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V91" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W91" s="24" t="s">
         <v>44</v>
@@ -10880,10 +10922,10 @@
         <v>81</v>
       </c>
       <c r="Z91" s="14" t="s">
-        <v>975</v>
+        <v>968</v>
       </c>
     </row>
-    <row r="92" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="17">
         <v>91</v>
       </c>
@@ -10891,34 +10933,34 @@
         <v>33</v>
       </c>
       <c r="C92" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="D92" s="16" t="s">
         <v>709</v>
       </c>
-      <c r="D92" s="16" t="s">
+      <c r="E92" s="16" t="s">
         <v>710</v>
-      </c>
-      <c r="E92" s="16" t="s">
-        <v>711</v>
       </c>
       <c r="F92" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J92" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L92" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M92" s="22" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="N92" s="22" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="T92" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V92" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W92" s="24" t="s">
         <v>44</v>
@@ -10930,10 +10972,10 @@
         <v>81</v>
       </c>
       <c r="Z92" s="14" t="s">
-        <v>976</v>
+        <v>969</v>
       </c>
     </row>
-    <row r="93" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="17">
         <v>92</v>
       </c>
@@ -10941,34 +10983,34 @@
         <v>33</v>
       </c>
       <c r="C93" s="7" t="s">
+        <v>711</v>
+      </c>
+      <c r="D93" s="16" t="s">
         <v>712</v>
       </c>
-      <c r="D93" s="16" t="s">
+      <c r="E93" s="16" t="s">
         <v>713</v>
-      </c>
-      <c r="E93" s="16" t="s">
-        <v>714</v>
       </c>
       <c r="F93" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J93" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L93" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M93" s="22" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="N93" s="22" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="T93" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V93" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W93" s="24" t="s">
         <v>44</v>
@@ -10980,10 +11022,10 @@
         <v>81</v>
       </c>
       <c r="Z93" s="14" t="s">
-        <v>977</v>
+        <v>970</v>
       </c>
     </row>
-    <row r="94" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="17">
         <v>93</v>
       </c>
@@ -10991,34 +11033,34 @@
         <v>33</v>
       </c>
       <c r="C94" s="7" t="s">
+        <v>714</v>
+      </c>
+      <c r="D94" s="16" t="s">
         <v>715</v>
       </c>
-      <c r="D94" s="16" t="s">
+      <c r="E94" s="16" t="s">
         <v>716</v>
-      </c>
-      <c r="E94" s="16" t="s">
-        <v>717</v>
       </c>
       <c r="F94" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J94" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L94" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M94" s="22" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="N94" s="22" t="s">
-        <v>921</v>
+        <v>918</v>
       </c>
       <c r="T94" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V94" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W94" s="24" t="s">
         <v>44</v>
@@ -11030,10 +11072,10 @@
         <v>81</v>
       </c>
       <c r="Z94" s="14" t="s">
-        <v>978</v>
+        <v>971</v>
       </c>
     </row>
-    <row r="95" spans="1:33" ht="45" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:33" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="17">
         <v>94</v>
       </c>
@@ -11041,22 +11083,22 @@
         <v>33</v>
       </c>
       <c r="C95" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="D95" s="16" t="s">
         <v>718</v>
       </c>
-      <c r="D95" s="16" t="s">
+      <c r="E95" s="16" t="s">
         <v>719</v>
-      </c>
-      <c r="E95" s="16" t="s">
-        <v>720</v>
       </c>
       <c r="F95" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J95" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L95" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M95" s="18" t="s">
         <v>51</v>
@@ -11074,7 +11116,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="96" spans="1:33" ht="90" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:33" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="17">
         <v>95</v>
       </c>
@@ -11082,34 +11124,34 @@
         <v>33</v>
       </c>
       <c r="C96" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="D96" s="16" t="s">
         <v>721</v>
       </c>
-      <c r="D96" s="16" t="s">
+      <c r="E96" s="16" t="s">
         <v>722</v>
-      </c>
-      <c r="E96" s="16" t="s">
-        <v>723</v>
       </c>
       <c r="F96" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J96" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L96" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M96" s="22" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="N96" s="22" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="T96" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V96" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W96" s="24" t="s">
         <v>44</v>
@@ -11121,10 +11163,10 @@
         <v>81</v>
       </c>
       <c r="Z96" s="14" t="s">
-        <v>979</v>
+        <v>972</v>
       </c>
     </row>
-    <row r="97" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="17">
         <v>96</v>
       </c>
@@ -11132,34 +11174,34 @@
         <v>33</v>
       </c>
       <c r="C97" s="7" t="s">
+        <v>723</v>
+      </c>
+      <c r="D97" s="16" t="s">
         <v>724</v>
       </c>
-      <c r="D97" s="16" t="s">
+      <c r="E97" s="16" t="s">
         <v>725</v>
-      </c>
-      <c r="E97" s="16" t="s">
-        <v>726</v>
       </c>
       <c r="F97" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J97" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L97" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M97" s="22" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="N97" s="22" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="T97" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V97" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W97" s="24" t="s">
         <v>44</v>
@@ -11171,10 +11213,10 @@
         <v>81</v>
       </c>
       <c r="Z97" s="14" t="s">
-        <v>980</v>
+        <v>973</v>
       </c>
     </row>
-    <row r="98" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="17">
         <v>97</v>
       </c>
@@ -11182,34 +11224,34 @@
         <v>33</v>
       </c>
       <c r="C98" s="7" t="s">
+        <v>726</v>
+      </c>
+      <c r="D98" s="16" t="s">
         <v>727</v>
       </c>
-      <c r="D98" s="16" t="s">
+      <c r="E98" s="16" t="s">
         <v>728</v>
-      </c>
-      <c r="E98" s="16" t="s">
-        <v>729</v>
       </c>
       <c r="F98" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J98" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L98" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M98" s="22" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="N98" s="22" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="T98" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V98" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W98" s="24" t="s">
         <v>44</v>
@@ -11221,10 +11263,10 @@
         <v>81</v>
       </c>
       <c r="Z98" s="14" t="s">
-        <v>981</v>
+        <v>974</v>
       </c>
     </row>
-    <row r="99" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="17">
         <v>98</v>
       </c>
@@ -11232,34 +11274,34 @@
         <v>33</v>
       </c>
       <c r="C99" s="7" t="s">
+        <v>729</v>
+      </c>
+      <c r="D99" s="16" t="s">
         <v>730</v>
       </c>
-      <c r="D99" s="16" t="s">
+      <c r="E99" s="16" t="s">
         <v>731</v>
-      </c>
-      <c r="E99" s="16" t="s">
-        <v>732</v>
       </c>
       <c r="F99" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J99" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L99" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M99" s="22" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="N99" s="22" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="T99" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V99" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W99" s="24" t="s">
         <v>44</v>
@@ -11271,10 +11313,10 @@
         <v>81</v>
       </c>
       <c r="Z99" s="14" t="s">
-        <v>982</v>
+        <v>975</v>
       </c>
     </row>
-    <row r="100" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="17">
         <v>99</v>
       </c>
@@ -11282,34 +11324,34 @@
         <v>33</v>
       </c>
       <c r="C100" s="7" t="s">
+        <v>732</v>
+      </c>
+      <c r="D100" s="16" t="s">
         <v>733</v>
       </c>
-      <c r="D100" s="16" t="s">
+      <c r="E100" s="16" t="s">
         <v>734</v>
-      </c>
-      <c r="E100" s="16" t="s">
-        <v>735</v>
       </c>
       <c r="F100" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J100" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L100" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M100" s="22" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="N100" s="22" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="T100" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V100" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W100" s="24" t="s">
         <v>44</v>
@@ -11321,10 +11363,10 @@
         <v>81</v>
       </c>
       <c r="Z100" s="14" t="s">
-        <v>983</v>
+        <v>976</v>
       </c>
     </row>
-    <row r="101" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="17">
         <v>100</v>
       </c>
@@ -11332,34 +11374,34 @@
         <v>33</v>
       </c>
       <c r="C101" s="7" t="s">
+        <v>735</v>
+      </c>
+      <c r="D101" s="16" t="s">
         <v>736</v>
       </c>
-      <c r="D101" s="16" t="s">
+      <c r="E101" s="16" t="s">
         <v>737</v>
-      </c>
-      <c r="E101" s="16" t="s">
-        <v>738</v>
       </c>
       <c r="F101" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J101" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L101" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M101" s="22" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="N101" s="22" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="T101" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V101" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W101" s="24" t="s">
         <v>44</v>
@@ -11371,10 +11413,10 @@
         <v>81</v>
       </c>
       <c r="Z101" s="14" t="s">
-        <v>984</v>
+        <v>977</v>
       </c>
     </row>
-    <row r="102" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="17">
         <v>101</v>
       </c>
@@ -11382,34 +11424,34 @@
         <v>33</v>
       </c>
       <c r="C102" s="7" t="s">
+        <v>738</v>
+      </c>
+      <c r="D102" s="16" t="s">
         <v>739</v>
       </c>
-      <c r="D102" s="16" t="s">
+      <c r="E102" s="16" t="s">
         <v>740</v>
-      </c>
-      <c r="E102" s="16" t="s">
-        <v>741</v>
       </c>
       <c r="F102" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J102" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L102" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M102" s="22" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="N102" s="22" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="T102" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V102" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W102" s="24" t="s">
         <v>44</v>
@@ -11421,10 +11463,10 @@
         <v>81</v>
       </c>
       <c r="Z102" s="14" t="s">
-        <v>985</v>
+        <v>978</v>
       </c>
     </row>
-    <row r="103" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="17">
         <v>102</v>
       </c>
@@ -11432,34 +11474,34 @@
         <v>33</v>
       </c>
       <c r="C103" s="7" t="s">
+        <v>741</v>
+      </c>
+      <c r="D103" s="16" t="s">
         <v>742</v>
       </c>
-      <c r="D103" s="16" t="s">
+      <c r="E103" s="16" t="s">
         <v>743</v>
-      </c>
-      <c r="E103" s="16" t="s">
-        <v>744</v>
       </c>
       <c r="F103" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J103" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L103" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M103" s="22" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="N103" s="22" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="T103" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V103" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W103" s="24" t="s">
         <v>44</v>
@@ -11471,10 +11513,10 @@
         <v>81</v>
       </c>
       <c r="Z103" s="14" t="s">
-        <v>986</v>
+        <v>979</v>
       </c>
     </row>
-    <row r="104" spans="1:26" ht="90" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:26" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="17">
         <v>103</v>
       </c>
@@ -11482,34 +11524,34 @@
         <v>33</v>
       </c>
       <c r="C104" s="7" t="s">
+        <v>744</v>
+      </c>
+      <c r="D104" s="16" t="s">
         <v>745</v>
       </c>
-      <c r="D104" s="16" t="s">
+      <c r="E104" s="16" t="s">
         <v>746</v>
-      </c>
-      <c r="E104" s="16" t="s">
-        <v>747</v>
       </c>
       <c r="F104" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J104" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L104" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M104" s="22" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="N104" s="22" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="T104" s="22" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="V104" s="22" t="s">
-        <v>992</v>
+        <v>985</v>
       </c>
       <c r="W104" s="24" t="s">
         <v>44</v>
@@ -11521,10 +11563,10 @@
         <v>81</v>
       </c>
       <c r="Z104" s="14" t="s">
-        <v>987</v>
+        <v>980</v>
       </c>
     </row>
-    <row r="105" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="17">
         <v>104</v>
       </c>
@@ -11532,24 +11574,24 @@
         <v>33</v>
       </c>
       <c r="C105" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="D105" s="16" t="s">
         <v>748</v>
       </c>
-      <c r="D105" s="16" t="s">
+      <c r="E105" s="16" t="s">
         <v>749</v>
-      </c>
-      <c r="E105" s="16" t="s">
-        <v>750</v>
       </c>
       <c r="F105" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J105" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L105" s="12" t="s">
-        <v>628</v>
-      </c>
-      <c r="M105" s="36" t="s">
+        <v>627</v>
+      </c>
+      <c r="M105" s="18" t="s">
         <v>51</v>
       </c>
       <c r="W105" s="16" t="s">
@@ -11565,7 +11607,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="106" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="17">
         <v>105</v>
       </c>
@@ -11573,22 +11615,22 @@
         <v>33</v>
       </c>
       <c r="C106" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="D106" s="16" t="s">
         <v>751</v>
       </c>
-      <c r="D106" s="16" t="s">
+      <c r="E106" s="16" t="s">
         <v>752</v>
-      </c>
-      <c r="E106" s="16" t="s">
-        <v>753</v>
       </c>
       <c r="F106" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J106" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L106" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M106" s="18" t="s">
         <v>51</v>
@@ -11606,7 +11648,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="107" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="17">
         <v>106</v>
       </c>
@@ -11614,22 +11656,22 @@
         <v>33</v>
       </c>
       <c r="C107" s="7" t="s">
+        <v>753</v>
+      </c>
+      <c r="D107" s="16" t="s">
         <v>754</v>
       </c>
-      <c r="D107" s="16" t="s">
+      <c r="E107" s="16" t="s">
         <v>755</v>
-      </c>
-      <c r="E107" s="16" t="s">
-        <v>756</v>
       </c>
       <c r="F107" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J107" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L107" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M107" s="18" t="s">
         <v>51</v>
@@ -11647,7 +11689,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="108" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="17">
         <v>107</v>
       </c>
@@ -11655,22 +11697,22 @@
         <v>33</v>
       </c>
       <c r="C108" s="7" t="s">
+        <v>756</v>
+      </c>
+      <c r="D108" s="16" t="s">
         <v>757</v>
       </c>
-      <c r="D108" s="16" t="s">
+      <c r="E108" s="16" t="s">
         <v>758</v>
-      </c>
-      <c r="E108" s="16" t="s">
-        <v>759</v>
       </c>
       <c r="F108" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J108" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L108" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M108" s="18" t="s">
         <v>51</v>
@@ -11688,7 +11730,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="109" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="17">
         <v>108</v>
       </c>
@@ -11696,22 +11738,22 @@
         <v>33</v>
       </c>
       <c r="C109" s="7" t="s">
+        <v>759</v>
+      </c>
+      <c r="D109" s="16" t="s">
         <v>760</v>
       </c>
-      <c r="D109" s="16" t="s">
+      <c r="E109" s="16" t="s">
         <v>761</v>
-      </c>
-      <c r="E109" s="16" t="s">
-        <v>762</v>
       </c>
       <c r="F109" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J109" s="7" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L109" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M109" s="18" t="s">
         <v>51</v>
@@ -11729,7 +11771,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="110" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="17">
         <v>109</v>
       </c>
@@ -11737,22 +11779,22 @@
         <v>33</v>
       </c>
       <c r="C110" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="D110" s="16" t="s">
         <v>763</v>
       </c>
-      <c r="D110" s="16" t="s">
+      <c r="E110" s="16" t="s">
         <v>764</v>
-      </c>
-      <c r="E110" s="16" t="s">
-        <v>765</v>
       </c>
       <c r="F110" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J110" s="7" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="L110" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M110" s="18" t="s">
         <v>51</v>
@@ -11770,7 +11812,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="111" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="17">
         <v>110</v>
       </c>
@@ -11778,22 +11820,22 @@
         <v>33</v>
       </c>
       <c r="C111" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="D111" s="16" t="s">
         <v>767</v>
       </c>
-      <c r="D111" s="16" t="s">
+      <c r="E111" s="16" t="s">
         <v>768</v>
-      </c>
-      <c r="E111" s="16" t="s">
-        <v>769</v>
       </c>
       <c r="F111" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J111" s="7" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="L111" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M111" s="18" t="s">
         <v>51</v>
@@ -11811,7 +11853,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="112" spans="1:26" ht="45" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:26" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="17">
         <v>111</v>
       </c>
@@ -11819,22 +11861,22 @@
         <v>33</v>
       </c>
       <c r="C112" s="7" t="s">
+        <v>770</v>
+      </c>
+      <c r="D112" s="16" t="s">
         <v>771</v>
       </c>
-      <c r="D112" s="16" t="s">
+      <c r="E112" s="16" t="s">
         <v>772</v>
-      </c>
-      <c r="E112" s="16" t="s">
-        <v>773</v>
       </c>
       <c r="F112" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J112" s="7" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="L112" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M112" s="18" t="s">
         <v>51</v>
@@ -11852,7 +11894,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="113" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="17">
         <v>112</v>
       </c>
@@ -11860,28 +11902,28 @@
         <v>33</v>
       </c>
       <c r="C113" s="7" t="s">
+        <v>773</v>
+      </c>
+      <c r="D113" s="16" t="s">
         <v>774</v>
       </c>
-      <c r="D113" s="16" t="s">
-        <v>775</v>
-      </c>
       <c r="E113" s="16" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="F113" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J113" s="7" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="L113" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M113" s="22" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="N113" s="22" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="O113" s="24"/>
       <c r="P113" s="24"/>
@@ -11889,10 +11931,10 @@
       <c r="R113" s="24"/>
       <c r="S113" s="24"/>
       <c r="T113" s="22" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="V113" s="22" t="s">
-        <v>935</v>
+        <v>995</v>
       </c>
       <c r="W113" s="16" t="s">
         <v>44</v>
@@ -11904,19 +11946,19 @@
         <v>81</v>
       </c>
       <c r="Z113" s="14" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="AA113" s="18" t="s">
+        <v>776</v>
+      </c>
+      <c r="AB113" s="36" t="s">
         <v>777</v>
       </c>
-      <c r="AB113" s="27" t="s">
-        <v>778</v>
-      </c>
       <c r="AC113" s="22" t="s">
-        <v>936</v>
+        <v>997</v>
       </c>
     </row>
-    <row r="114" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="17">
         <v>113</v>
       </c>
@@ -11924,28 +11966,28 @@
         <v>33</v>
       </c>
       <c r="C114" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="D114" s="16" t="s">
         <v>779</v>
       </c>
-      <c r="D114" s="16" t="s">
-        <v>780</v>
-      </c>
       <c r="E114" s="16" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="F114" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J114" s="7" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="L114" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M114" s="22" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="N114" s="22" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="O114" s="24"/>
       <c r="P114" s="24"/>
@@ -11953,10 +11995,10 @@
       <c r="R114" s="24"/>
       <c r="S114" s="24"/>
       <c r="T114" s="22" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="V114" s="22" t="s">
-        <v>935</v>
+        <v>994</v>
       </c>
       <c r="W114" s="16" t="s">
         <v>44</v>
@@ -11968,16 +12010,16 @@
         <v>81</v>
       </c>
       <c r="Z114" s="14" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="AA114" s="18" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="AC114" s="22" t="s">
-        <v>936</v>
+        <v>998</v>
       </c>
     </row>
-    <row r="115" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:29" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="17">
         <v>114</v>
       </c>
@@ -11985,28 +12027,28 @@
         <v>33</v>
       </c>
       <c r="C115" s="7" t="s">
+        <v>782</v>
+      </c>
+      <c r="D115" s="16" t="s">
         <v>783</v>
       </c>
-      <c r="D115" s="16" t="s">
-        <v>784</v>
-      </c>
       <c r="E115" s="16" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="F115" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J115" s="7" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="L115" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="M115" s="22" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="N115" s="22" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="O115" s="24"/>
       <c r="P115" s="24"/>
@@ -12014,10 +12056,10 @@
       <c r="R115" s="24"/>
       <c r="S115" s="24"/>
       <c r="T115" s="22" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="V115" s="22" t="s">
-        <v>935</v>
+        <v>996</v>
       </c>
       <c r="W115" s="16" t="s">
         <v>44</v>
@@ -12029,19 +12071,19 @@
         <v>81</v>
       </c>
       <c r="Z115" s="14" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="AA115" s="18" t="s">
+        <v>784</v>
+      </c>
+      <c r="AB115" s="18" t="s">
         <v>785</v>
       </c>
-      <c r="AB115" s="18" t="s">
-        <v>786</v>
-      </c>
       <c r="AC115" s="22" t="s">
-        <v>936</v>
+        <v>999</v>
       </c>
     </row>
-    <row r="116" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="17">
         <v>115</v>
       </c>
@@ -12049,19 +12091,19 @@
         <v>33</v>
       </c>
       <c r="C116" s="7" t="s">
+        <v>786</v>
+      </c>
+      <c r="D116" s="16" t="s">
         <v>787</v>
       </c>
-      <c r="D116" s="16" t="s">
-        <v>788</v>
-      </c>
       <c r="E116" s="16" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="F116" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J116" s="7" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="M116" s="18" t="s">
         <v>51</v>
@@ -12079,7 +12121,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="117" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="17">
         <v>116</v>
       </c>
@@ -12087,19 +12129,19 @@
         <v>33</v>
       </c>
       <c r="C117" s="7" t="s">
+        <v>789</v>
+      </c>
+      <c r="D117" s="16" t="s">
         <v>790</v>
       </c>
-      <c r="D117" s="16" t="s">
-        <v>791</v>
-      </c>
       <c r="E117" s="16" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="F117" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J117" s="7" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="M117" s="18" t="s">
         <v>51</v>
@@ -12117,7 +12159,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="118" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:29" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="17">
         <v>117</v>
       </c>
@@ -12125,40 +12167,40 @@
         <v>33</v>
       </c>
       <c r="C118" s="7" t="s">
+        <v>792</v>
+      </c>
+      <c r="D118" s="16" t="s">
         <v>793</v>
       </c>
-      <c r="D118" s="16" t="s">
-        <v>794</v>
-      </c>
       <c r="E118" s="16" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="F118" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J118" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="M118" s="18" t="s">
         <v>795</v>
       </c>
-      <c r="M118" s="18" t="s">
+      <c r="N118" s="18" t="s">
         <v>796</v>
       </c>
-      <c r="N118" s="18" t="s">
+      <c r="O118" s="16" t="s">
         <v>797</v>
       </c>
-      <c r="O118" s="16" t="s">
+      <c r="P118" s="16" t="s">
         <v>798</v>
       </c>
-      <c r="P118" s="16" t="s">
+      <c r="Q118" s="16" t="s">
         <v>799</v>
-      </c>
-      <c r="Q118" s="16" t="s">
-        <v>800</v>
       </c>
       <c r="S118" s="16" t="s">
         <v>104</v>
       </c>
       <c r="T118" s="18" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="W118" s="16" t="s">
         <v>44</v>
@@ -12170,13 +12212,13 @@
         <v>81</v>
       </c>
       <c r="Z118" s="14" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="AC118" s="22" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
-    <row r="119" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="17">
         <v>118</v>
       </c>
@@ -12184,19 +12226,19 @@
         <v>33</v>
       </c>
       <c r="C119" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="D119" s="16" t="s">
         <v>802</v>
       </c>
-      <c r="D119" s="16" t="s">
-        <v>803</v>
-      </c>
       <c r="E119" s="16" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="F119" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J119" s="7" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="M119" s="18" t="s">
         <v>51</v>
@@ -12214,7 +12256,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="120" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="17">
         <v>119</v>
       </c>
@@ -12222,22 +12264,22 @@
         <v>33</v>
       </c>
       <c r="C120" s="7" t="s">
+        <v>804</v>
+      </c>
+      <c r="D120" s="16" t="s">
         <v>805</v>
       </c>
-      <c r="D120" s="16" t="s">
-        <v>806</v>
-      </c>
       <c r="E120" s="16" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="F120" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J120" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="K120" s="7" t="s">
         <v>807</v>
-      </c>
-      <c r="K120" s="7" t="s">
-        <v>808</v>
       </c>
       <c r="M120" s="18" t="s">
         <v>51</v>
@@ -12255,7 +12297,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="121" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="17">
         <v>120</v>
       </c>
@@ -12263,19 +12305,19 @@
         <v>33</v>
       </c>
       <c r="C121" s="7" t="s">
+        <v>808</v>
+      </c>
+      <c r="D121" s="16" t="s">
         <v>809</v>
       </c>
-      <c r="D121" s="16" t="s">
-        <v>810</v>
-      </c>
       <c r="E121" s="16" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="F121" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J121" s="7" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="M121" s="18" t="s">
         <v>51</v>
@@ -12293,7 +12335,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="122" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:29" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="17">
         <v>121</v>
       </c>
@@ -12301,19 +12343,19 @@
         <v>33</v>
       </c>
       <c r="C122" s="7" t="s">
+        <v>810</v>
+      </c>
+      <c r="D122" s="16" t="s">
         <v>811</v>
       </c>
-      <c r="D122" s="16" t="s">
-        <v>812</v>
-      </c>
       <c r="E122" s="16" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="F122" s="7" t="s">
         <v>63</v>
       </c>
       <c r="J122" s="7" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="M122" s="18" t="s">
         <v>51</v>
@@ -12332,7 +12374,27 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG122" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" ref="A1:AG122" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="25">
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x14">
+          <filters>
+            <x14:filter val="case_when(_x000a_(rowSums(mutate(.,_x000a_temp_B10Q12A = case_when(B10Q12A == 1 ~ 0*5;_x000a_B10Q12A == 2 ~ 0.5*5;_x000a_B10Q12A == 3 ~ 1.5*5;_x000a_B10Q12A == 4 ~ 2.5*5;_x000a_B10Q12A == 5 ~ 3.5*5;_x000a_B10Q12A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q12B = case_when(B10Q12B == 1 ~ 0.5*2;_x000a_B10Q12B == 2 ~ 0.5*2;_x000a_B10Q12B == 3 ~ 1.5*2;_x000a_B10Q12B == 4 ~ 2.5*2;_x000a_B10Q12B == 5 ~ 3.5*2;_x000a_B10Q12B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q12A, temp_B10Q12B), na.rm = FALSE)/7) &lt; 1 ~ 1L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q12A = case_when(B10Q12A == 1 ~ 0*5;_x000a_B10Q12A == 2 ~ 0.5*5;_x000a_B10Q12A == 3 ~ 1.5*5;_x000a_B10Q12A == 4 ~ 2.5*5;_x000a_B10Q12A == 5 ~ 3.5*5;_x000a_B10Q12A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q12B = case_when(B10Q12B == 1 ~ 0.5*2;_x000a_B10Q12B == 2 ~ 0.5*2;_x000a_B10Q12B == 3 ~ 1.5*2;_x000a_B10Q12B == 4 ~ 2.5*2;_x000a_B10Q12B == 5 ~ 3.5*2;_x000a_B10Q12B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q12A, temp_B10Q12B), na.rm = FALSE)/7) &gt;= 1 &amp;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q12A = case_when(B10Q12A == 1 ~ 0*5;_x000a_B10Q12A == 2 ~ 0.5*5;_x000a_B10Q12A == 3 ~ 1.5*5;_x000a_B10Q12A == 4 ~ 2.5*5;_x000a_B10Q12A == 5 ~ 3.5*5;_x000a_B10Q12A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q12B = case_when(B10Q12B == 1 ~ 0.5*2;_x000a_B10Q12B == 2 ~ 0.5*2;_x000a_B10Q12B == 3 ~ 1.5*2;_x000a_B10Q12B == 4 ~ 2.5*2;_x000a_B10Q12B == 5 ~ 3.5*2;_x000a_B10Q12B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q12A, temp_B10Q12B), na.rm = FALSE)/7) &lt;= 3 ~ 2L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q12A = case_when(B10Q12A == 1 ~ 0*5;_x000a_B10Q12A == 2 ~ 0.5*5;_x000a_B10Q12A == 3 ~ 1.5*5;_x000a_B10Q12A == 4 ~ 2.5*5;_x000a_B10Q12A == 5 ~ 3.5*5;_x000a_B10Q12A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q12B = case_when(B10Q12B == 1 ~ 0.5*2;_x000a_B10Q12B == 2 ~ 0.5*2;_x000a_B10Q12B == 3 ~ 1.5*2;_x000a_B10Q12B == 4 ~ 2.5*2;_x000a_B10Q12B == 5 ~ 3.5*2;_x000a_B10Q12B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q12A, temp_B10Q12B), na.rm = FALSE)/7) &gt; 3 ~ 3L; _x000a_ELSE ~ NA_integer_)_x000a_"/>
+            <x14:filter val="case_when(_x000a_(rowSums(mutate(.,_x000a_temp_B10Q13A = case_when(B10Q13A == 1 ~ 0*5;_x000a_B10Q13A == 2 ~ 0.5*5;_x000a_B10Q13A == 3 ~ 1.5*5;_x000a_B10Q13A == 4 ~ 2.5*5;_x000a_B10Q13A == 5 ~ 3.5*5;_x000a_B10Q13A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q13B = case_when(B10Q13B == 1 ~ 0.5*2;_x000a_B10Q13B == 2 ~ 0.5*2;_x000a_B10Q13B == 3 ~ 1.5*2;_x000a_B10Q13B == 4 ~ 2.5*2;_x000a_B10Q13B == 5 ~ 3.5*2;_x000a_B10Q13B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q13A, temp_B10Q13B), na.rm = FALSE)/7) &lt; 1 ~ 1L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q13A = case_when(B10Q13A == 1 ~ 0*5;_x000a_B10Q13A == 2 ~ 0.5*5;_x000a_B10Q13A == 3 ~ 1.5*5;_x000a_B10Q13A == 4 ~ 2.5*5;_x000a_B10Q13A == 5 ~ 3.5*5;_x000a_B10Q13A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q13B = case_when(B10Q13B == 1 ~ 0.5*2;_x000a_B10Q13B == 2 ~ 0.5*2;_x000a_B10Q13B == 3 ~ 1.5*2;_x000a_B10Q13B == 4 ~ 2.5*2;_x000a_B10Q13B == 5 ~ 3.5*2;_x000a_B10Q13B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q13A, temp_B10Q13B), na.rm = FALSE)/7) &gt;= 1 &amp;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q13A = case_when(B10Q13A == 1 ~ 0*5;_x000a_B10Q13A == 2 ~ 0.5*5;_x000a_B10Q13A == 3 ~ 1.5*5;_x000a_B10Q13A == 4 ~ 2.5*5;_x000a_B10Q13A == 5 ~ 3.5*5;_x000a_B10Q13A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q13B = case_when(B10Q13B == 1 ~ 0.5*2;_x000a_B10Q13B == 2 ~ 0.5*2;_x000a_B10Q13B == 3 ~ 1.5*2;_x000a_B10Q13B == 4 ~ 2.5*2;_x000a_B10Q13B == 5 ~ 3.5*2;_x000a_B10Q13B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q13A, temp_B10Q13B), na.rm = FALSE)/7) &lt;= 3 ~ 2L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q13A = case_when(B10Q13A == 1 ~ 0*5;_x000a_B10Q13A == 2 ~ 0.5*5;_x000a_B10Q13A == 3 ~ 1.5*5;_x000a_B10Q13A == 4 ~ 2.5*5;_x000a_B10Q13A == 5 ~ 3.5*5;_x000a_B10Q13A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q13B = case_when(B10Q13B == 1 ~ 0.5*2;_x000a_B10Q13B == 2 ~ 0.5*2;_x000a_B10Q13B == 3 ~ 1.5*2;_x000a_B10Q13B == 4 ~ 2.5*2;_x000a_B10Q13B == 5 ~ 3.5*2;_x000a_B10Q13B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q13A, temp_B10Q13B), na.rm = FALSE)/7) &gt; 3 ~ 3L; _x000a_ELSE ~ NA_integer_)_x000a_"/>
+            <x14:filter val="case_when(_x000a_(rowSums(mutate(.,_x000a_temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;_x000a_B10Q15A == 2 ~ 0.5*5;_x000a_B10Q15A == 3 ~ 1.5*5;_x000a_B10Q15A == 4 ~ 2.5*5;_x000a_B10Q15A == 5 ~ 3.5*5;_x000a_B10Q15A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;_x000a_B10Q15B == 2 ~ 0.5*2;_x000a_B10Q15B == 3 ~ 1.5*2;_x000a_B10Q15B == 4 ~ 2.5*2;_x000a_B10Q15B == 5 ~ 3.5*2;_x000a_B10Q15B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt; 1 ~ 1L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;_x000a_B10Q15A == 2 ~ 0.5*5;_x000a_B10Q15A == 3 ~ 1.5*5;_x000a_B10Q15A == 4 ~ 2.5*5;_x000a_B10Q15A == 5 ~ 3.5*5;_x000a_B10Q15A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;_x000a_B10Q15B == 2 ~ 0.5*2;_x000a_B10Q15B == 3 ~ 1.5*2;_x000a_B10Q15B == 4 ~ 2.5*2;_x000a_B10Q15B == 5 ~ 3.5*2;_x000a_B10Q15B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt;= 1 &amp;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;_x000a_B10Q15A == 2 ~ 0.5*5;_x000a_B10Q15A == 3 ~ 1.5*5;_x000a_B10Q15A == 4 ~ 2.5*5;_x000a_B10Q15A == 5 ~ 3.5*5;_x000a_B10Q15A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;_x000a_B10Q15B == 2 ~ 0.5*2;_x000a_B10Q15B == 3 ~ 1.5*2;_x000a_B10Q15B == 4 ~ 2.5*2;_x000a_B10Q15B == 5 ~ 3.5*2;_x000a_B10Q15B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &lt;= 3 ~ 2L;_x000a_(rowSums(mutate(.,_x000a_temp_B10Q15A = case_when(B10Q15A == 1 ~ 0*5;_x000a_B10Q15A == 2 ~ 0.5*5;_x000a_B10Q15A == 3 ~ 1.5*5;_x000a_B10Q15A == 4 ~ 2.5*5;_x000a_B10Q15A == 5 ~ 3.5*5;_x000a_B10Q15A == 6 ~ 4*5;_x000a_ELSE ~ NA_real_),_x000a__x000a_temp_B10Q15B = case_when(B10Q15B == 1 ~ 0.5*2;_x000a_B10Q15B == 2 ~ 0.5*2;_x000a_B10Q15B == 3 ~ 1.5*2;_x000a_B10Q15B == 4 ~ 2.5*2;_x000a_B10Q15B == 5 ~ 3.5*2;_x000a_B10Q15B == 6 ~ 4*2;_x000a_ELSE ~ NA_real_)) %&gt;%_x000a_select(temp_B10Q15A, temp_B10Q15B), na.rm = FALSE)/7) &gt; 3 ~ 3L; _x000a_ELSE ~ NA_integer_)_x000a_"/>
+            <x14:filter val="case_when(_x000a_rowSums(mutate(.,_x000a_temp_B10Q2A = if_else(!B10Q2A %in% c(1, 2, 3), NA, 1), _x000a_temp_B10Q2B = if_else(!B10Q2B %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2C = if_else(!B10Q2C %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2D = if_else(!B10Q2D %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2E = if_else(!B10Q2E %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2F = if_else(!B10Q2F %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2G = if_else(!B10Q2G %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2H = if_else(!B10Q2H %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2I = if_else(!B10Q2I %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2J = if_else(!B10Q2J %in% c(1, 2, 3), NA, 1)) %&gt;%_x000a_select(temp_B10Q2A, temp_B10Q2B, temp_B10Q2C, temp_B10Q2D, temp_B10Q2E,_x000a_temp_B10Q2F, temp_B10Q2G, temp_B10Q2H, temp_B10Q2I, temp_B10Q2J), _x000a_na.rm = TRUE) &lt; 5 ~ NA_real_ ; _x000a_BD10PHHE &gt;= 0 ~ as.numeric(BD10PHHE);_x000a_ELSE ~ NA_real_)"/>
+            <x14:filter val="rowSums(mutate(.,_x000a_temp_B10Q2A = if_else(!B10Q2A %in% c(1, 2, 3), NA, 1), _x000a_temp_B10Q2B = if_else(!B10Q2B %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2C = if_else(!B10Q2C %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2D = if_else(!B10Q2D %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2E = if_else(!B10Q2E %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2F = if_else(!B10Q2F %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2G = if_else(!B10Q2G %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2H = if_else(!B10Q2H %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2I = if_else(!B10Q2I %in% c(1, 2, 3), NA, 1),_x000a_temp_B10Q2J = if_else(!B10Q2J %in% c(1, 2, 3), NA, 1)) %&gt;%_x000a_select(temp_B10Q2A, temp_B10Q2B, temp_B10Q2C, temp_B10Q2D, temp_B10Q2E,_x000a_temp_B10Q2F, temp_B10Q2G, temp_B10Q2H, temp_B10Q2I, temp_B10Q2J), _x000a_na.rm = TRUE)"/>
+          </filters>
+        </mc:Choice>
+        <mc:Fallback>
+          <customFilters>
+            <customFilter val=""/>
+            <customFilter operator="notEqual" val=" "/>
+          </customFilters>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S75" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>#REF!</formula1>

</xml_diff>